<commit_message>
docs: actualización seguimiento casosde prueba"
</commit_message>
<xml_diff>
--- a/Plan_de_pruebas_analisis.xlsx
+++ b/Plan_de_pruebas_analisis.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11580" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="12180" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Back" sheetId="1" r:id="rId1"/>
@@ -813,7 +813,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -885,13 +885,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1004,7 +997,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="44">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1109,12 +1102,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1145,25 +1132,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1205,18 +1174,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1248,18 +1205,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1505,99 +1450,117 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1606,37 +1569,19 @@
     <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>

</xml_diff>

<commit_message>
docs; actualización casos filtros
</commit_message>
<xml_diff>
--- a/Plan_de_pruebas_analisis.xlsx
+++ b/Plan_de_pruebas_analisis.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="11580" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Back" sheetId="1" r:id="rId1"/>
     <sheet name="Front" sheetId="2" r:id="rId2"/>
     <sheet name="Escenarios" sheetId="3" r:id="rId3"/>
-    <sheet name="Hoja4" sheetId="4" r:id="rId4"/>
+    <sheet name="Filtros" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="219">
   <si>
     <t>BackEnd</t>
   </si>
@@ -717,6 +717,69 @@
   </si>
   <si>
     <t>Filtros productos</t>
+  </si>
+  <si>
+    <t>/api/v1/products/?title</t>
+  </si>
+  <si>
+    <t>Consulta la lista de todos los productos  por mismo titulo</t>
+  </si>
+  <si>
+    <t>* Validar que el servicio retorne todos los productos al buscar por un titulo especifico</t>
+  </si>
+  <si>
+    <t>Lista de productos</t>
+  </si>
+  <si>
+    <t>* Numero total de productos.
+* Validar contrato de la respuesta para cada elemento. 
+* Validar codigo de estado.
+* Validar que en la respuesta los productos esten realacionado con el titulo buscado</t>
+  </si>
+  <si>
+    <t>/api/v1/products/?price</t>
+  </si>
+  <si>
+    <t>Consulta la lista de todos los productos por el precio</t>
+  </si>
+  <si>
+    <t>* Validar que el servicio retorne todos los productos al buscar por un precio especifico</t>
+  </si>
+  <si>
+    <t>* Numero total de productos.
+* Validar contrato de la respuesta para cada elemento. 
+* Validar codigo de estado.
+* Validar que en la respuesta los productos esten realacionado con el precio  buscado</t>
+  </si>
+  <si>
+    <t>/api/v1/products/?price_min&amp;price_max</t>
+  </si>
+  <si>
+    <t>Consulta la lista de todos los productos por precio dentro de un rango dado</t>
+  </si>
+  <si>
+    <t>/api/v1/products/?price_max&amp;price_min</t>
+  </si>
+  <si>
+    <t>* Validar que el servicio retorne todos los productos al buscar por un precio mayor y menor</t>
+  </si>
+  <si>
+    <t>/api/v1/products/?categoryId</t>
+  </si>
+  <si>
+    <t>Consulta la lista de todos los productos realciandos por categoria Id</t>
+  </si>
+  <si>
+    <t>* Validar que el servicio retorne todos los productos al buscar por categoria id</t>
+  </si>
+  <si>
+    <t>* Numero total de productos.
+* Validar contrato de la respuesta para cada elemento. 
+* Validar codigo de estado.
+* Validar que en la respuesta los productos esten realacionado con el id  buscado</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t>[GET] https://api.escuelajs.co/api/v1/products</t>
@@ -997,7 +1060,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1019,6 +1082,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1085,6 +1154,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1469,7 +1544,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1493,14 +1568,14 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1509,83 +1584,83 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1604,11 +1679,15 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="22" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="22" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1623,6 +1702,18 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1632,19 +1723,7 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1653,28 +1732,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1695,79 +1774,79 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="24" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="24" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="24" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="9" xfId="18" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="24" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="9" xfId="18" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="9" xfId="18" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="9" xfId="18" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="4" xfId="23" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="23" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="23" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="4" xfId="23" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="23" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="23" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="23" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="23" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="23" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="23" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1788,16 +1867,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="2" xfId="24" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="24" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="3" xfId="24" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="3" xfId="24" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="4" xfId="24" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="4" xfId="24" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1812,7 +1891,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1836,13 +1915,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="23" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="18" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="18" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="18" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="18" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="23" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="23" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1854,7 +1933,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1875,27 +1954,48 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="23" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="3" xfId="23" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="23" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="23" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="3" xfId="23" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="23" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="3" xfId="23" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="3" xfId="23" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="4" xfId="23" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="4" xfId="23" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1909,6 +2009,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2251,7 +2354,7 @@
       </c>
     </row>
     <row r="3" ht="90" spans="1:2">
-      <c r="B3" s="111" t="s">
+      <c r="B3" s="120" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2301,7 +2404,7 @@
       </c>
     </row>
     <row r="17" spans="2:2">
-      <c r="B17" s="112" t="s">
+      <c r="B17" s="121" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2340,22 +2443,22 @@
       <c r="A2" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="107" t="s">
+      <c r="B2" s="116" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" ht="30" spans="1:2">
-      <c r="B3" s="108" t="s">
+      <c r="B3" s="117" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" ht="30" spans="1:2">
-      <c r="B4" s="108" t="s">
+      <c r="B4" s="117" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="B9" s="109" t="s">
+      <c r="B9" s="118" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2380,27 +2483,27 @@
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="B16" s="110" t="s">
+      <c r="B16" s="119" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="17" ht="45" spans="2:2">
-      <c r="B17" s="111" t="s">
+      <c r="B17" s="120" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="18" ht="30" spans="2:2">
-      <c r="B18" s="111" t="s">
+      <c r="B18" s="120" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="19" ht="30" spans="2:2">
-      <c r="B19" s="108" t="s">
+      <c r="B19" s="117" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="20" ht="30" spans="2:2">
-      <c r="B20" s="111" t="s">
+      <c r="B20" s="120" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2413,1821 +2516,1996 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Y55"/>
+  <dimension ref="A1:Y59"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="19" width="11.4285714285714" style="12"/>
-    <col min="20" max="23" width="11.4285714285714" style="13"/>
+    <col min="1" max="19" width="11.4285714285714" style="14"/>
+    <col min="20" max="23" width="11.4285714285714" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
-      <c r="P1" s="14"/>
-      <c r="Q1" s="14"/>
-      <c r="R1" s="14"/>
-      <c r="S1" s="14"/>
-      <c r="T1" s="14"/>
-      <c r="U1" s="14"/>
-      <c r="V1" s="14"/>
-      <c r="W1" s="14"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="16"/>
+      <c r="T1" s="16"/>
+      <c r="U1" s="16"/>
+      <c r="V1" s="16"/>
+      <c r="W1" s="16"/>
     </row>
     <row r="2" spans="1:23">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="16"/>
-      <c r="M2" s="16"/>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
-      <c r="T2" s="16"/>
-      <c r="U2" s="16"/>
-      <c r="V2" s="16"/>
-      <c r="W2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="18"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="18"/>
+      <c r="S2" s="18"/>
+      <c r="T2" s="18"/>
+      <c r="U2" s="18"/>
+      <c r="V2" s="18"/>
+      <c r="W2" s="19"/>
     </row>
     <row r="3" spans="1:23">
-      <c r="A3" s="18"/>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18" t="s">
+      <c r="A3" s="20"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="19" t="s">
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I3" s="20"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="19" t="s">
+      <c r="I3" s="22"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="L3" s="20"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="19" t="s">
+      <c r="L3" s="22"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="O3" s="20"/>
-      <c r="P3" s="21"/>
-      <c r="Q3" s="19" t="s">
+      <c r="O3" s="22"/>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="R3" s="20"/>
-      <c r="S3" s="21"/>
-      <c r="T3" s="22" t="s">
+      <c r="R3" s="22"/>
+      <c r="S3" s="23"/>
+      <c r="T3" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
+      <c r="U3" s="24"/>
+      <c r="V3" s="24"/>
+      <c r="W3" s="24"/>
     </row>
     <row r="4" ht="106.5" customHeight="1" spans="1:23">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="25" t="s">
+      <c r="B4" s="26"/>
+      <c r="C4" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
-      <c r="H4" s="27" t="s">
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="I4" s="28"/>
-      <c r="J4" s="25"/>
-      <c r="K4" s="29" t="s">
+      <c r="I4" s="30"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="L4" s="29"/>
-      <c r="M4" s="29"/>
-      <c r="N4" s="26">
+      <c r="L4" s="31"/>
+      <c r="M4" s="31"/>
+      <c r="N4" s="28">
         <v>201</v>
       </c>
-      <c r="O4" s="26"/>
-      <c r="P4" s="26"/>
-      <c r="Q4" s="26" t="s">
+      <c r="O4" s="28"/>
+      <c r="P4" s="28"/>
+      <c r="Q4" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="R4" s="26"/>
-      <c r="S4" s="26"/>
-      <c r="T4" s="30" t="s">
+      <c r="R4" s="28"/>
+      <c r="S4" s="28"/>
+      <c r="T4" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="U4" s="31"/>
-      <c r="V4" s="31"/>
-      <c r="W4" s="32"/>
+      <c r="U4" s="33"/>
+      <c r="V4" s="33"/>
+      <c r="W4" s="34"/>
     </row>
     <row r="5" ht="123" customHeight="1" spans="1:23">
-      <c r="A5" s="33"/>
-      <c r="B5" s="34"/>
-      <c r="C5" s="35" t="s">
+      <c r="A5" s="35"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="37" t="s">
         <v>40</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
-      <c r="H5" s="36" t="s">
+      <c r="H5" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
-      <c r="K5" s="36" t="s">
+      <c r="I5" s="38"/>
+      <c r="J5" s="38"/>
+      <c r="K5" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="L5" s="36"/>
-      <c r="M5" s="36"/>
+      <c r="L5" s="38"/>
+      <c r="M5" s="38"/>
       <c r="N5" s="4">
         <v>400</v>
       </c>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
-      <c r="Q5" s="36" t="s">
+      <c r="Q5" s="38" t="s">
         <v>47</v>
       </c>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
-      <c r="T5" s="37" t="s">
+      <c r="T5" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="U5" s="38"/>
-      <c r="V5" s="38"/>
-      <c r="W5" s="38"/>
+      <c r="U5" s="40"/>
+      <c r="V5" s="40"/>
+      <c r="W5" s="40"/>
     </row>
     <row r="6" ht="154.5" customHeight="1" spans="1:23">
-      <c r="A6" s="33"/>
-      <c r="B6" s="34"/>
-      <c r="C6" s="35" t="s">
+      <c r="A6" s="35"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="37" t="s">
         <v>40</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="36" t="s">
+      <c r="H6" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="I6" s="36"/>
-      <c r="J6" s="36"/>
-      <c r="K6" s="36" t="s">
+      <c r="I6" s="38"/>
+      <c r="J6" s="38"/>
+      <c r="K6" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="L6" s="36"/>
-      <c r="M6" s="36"/>
+      <c r="L6" s="38"/>
+      <c r="M6" s="38"/>
       <c r="N6" s="4">
         <v>400</v>
       </c>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
-      <c r="Q6" s="36" t="s">
+      <c r="Q6" s="38" t="s">
         <v>51</v>
       </c>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
-      <c r="T6" s="37" t="s">
+      <c r="T6" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="U6" s="38"/>
-      <c r="V6" s="38"/>
-      <c r="W6" s="38"/>
+      <c r="U6" s="40"/>
+      <c r="V6" s="40"/>
+      <c r="W6" s="40"/>
     </row>
     <row r="7" ht="197.25" customHeight="1" spans="1:23">
-      <c r="A7" s="33"/>
-      <c r="B7" s="34"/>
-      <c r="C7" s="35" t="s">
+      <c r="A7" s="35"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="37" t="s">
         <v>40</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
-      <c r="H7" s="36" t="s">
+      <c r="H7" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="I7" s="36"/>
-      <c r="J7" s="36"/>
-      <c r="K7" s="36" t="s">
+      <c r="I7" s="38"/>
+      <c r="J7" s="38"/>
+      <c r="K7" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="L7" s="36"/>
-      <c r="M7" s="36"/>
+      <c r="L7" s="38"/>
+      <c r="M7" s="38"/>
       <c r="N7" s="4">
         <v>400</v>
       </c>
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
-      <c r="Q7" s="39" t="s">
+      <c r="Q7" s="41" t="s">
         <v>54</v>
       </c>
-      <c r="R7" s="40"/>
-      <c r="S7" s="40"/>
-      <c r="T7" s="37" t="s">
+      <c r="R7" s="42"/>
+      <c r="S7" s="42"/>
+      <c r="T7" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="U7" s="38"/>
-      <c r="V7" s="38"/>
-      <c r="W7" s="38"/>
+      <c r="U7" s="40"/>
+      <c r="V7" s="40"/>
+      <c r="W7" s="40"/>
     </row>
     <row r="8" ht="133.5" customHeight="1" spans="1:23">
-      <c r="A8" s="33"/>
-      <c r="B8" s="34"/>
-      <c r="C8" s="35" t="s">
+      <c r="A8" s="35"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="37" t="s">
         <v>40</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
-      <c r="H8" s="36" t="s">
+      <c r="H8" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="I8" s="36"/>
-      <c r="J8" s="36"/>
-      <c r="K8" s="36" t="s">
+      <c r="I8" s="38"/>
+      <c r="J8" s="38"/>
+      <c r="K8" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="L8" s="36"/>
-      <c r="M8" s="36"/>
+      <c r="L8" s="38"/>
+      <c r="M8" s="38"/>
       <c r="N8" s="4">
         <v>400</v>
       </c>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
-      <c r="Q8" s="36" t="s">
+      <c r="Q8" s="38" t="s">
         <v>57</v>
       </c>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
-      <c r="T8" s="41" t="s">
+      <c r="T8" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="U8" s="42"/>
-      <c r="V8" s="42"/>
-      <c r="W8" s="42"/>
+      <c r="U8" s="44"/>
+      <c r="V8" s="44"/>
+      <c r="W8" s="44"/>
     </row>
     <row r="9" ht="137.25" customHeight="1" spans="1:23">
-      <c r="A9" s="33"/>
-      <c r="B9" s="34"/>
-      <c r="C9" s="35" t="s">
+      <c r="A9" s="35"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="37" t="s">
         <v>40</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
-      <c r="H9" s="36" t="s">
+      <c r="H9" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="I9" s="36"/>
-      <c r="J9" s="36"/>
-      <c r="K9" s="36" t="s">
+      <c r="I9" s="38"/>
+      <c r="J9" s="38"/>
+      <c r="K9" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="L9" s="36"/>
-      <c r="M9" s="36"/>
+      <c r="L9" s="38"/>
+      <c r="M9" s="38"/>
       <c r="N9" s="4">
         <v>400</v>
       </c>
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
-      <c r="Q9" s="36" t="s">
+      <c r="Q9" s="38" t="s">
         <v>60</v>
       </c>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
-      <c r="T9" s="41" t="s">
+      <c r="T9" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="U9" s="42"/>
-      <c r="V9" s="42"/>
-      <c r="W9" s="42"/>
+      <c r="U9" s="44"/>
+      <c r="V9" s="44"/>
+      <c r="W9" s="44"/>
     </row>
     <row r="10" ht="174" customHeight="1" spans="1:23">
       <c r="A10" s="4" t="s">
         <v>61</v>
       </c>
       <c r="B10" s="4"/>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26" t="s">
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="I10" s="26"/>
-      <c r="J10" s="26"/>
-      <c r="K10" s="29" t="s">
+      <c r="I10" s="28"/>
+      <c r="J10" s="28"/>
+      <c r="K10" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="L10" s="29"/>
-      <c r="M10" s="29"/>
-      <c r="N10" s="43">
+      <c r="L10" s="31"/>
+      <c r="M10" s="31"/>
+      <c r="N10" s="45">
         <v>200</v>
       </c>
-      <c r="O10" s="44"/>
-      <c r="P10" s="45"/>
-      <c r="Q10" s="26" t="s">
+      <c r="O10" s="46"/>
+      <c r="P10" s="47"/>
+      <c r="Q10" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="R10" s="26"/>
-      <c r="S10" s="26"/>
-      <c r="T10" s="46" t="s">
+      <c r="R10" s="28"/>
+      <c r="S10" s="28"/>
+      <c r="T10" s="48" t="s">
         <v>66</v>
       </c>
-      <c r="U10" s="46"/>
-      <c r="V10" s="46"/>
-      <c r="W10" s="46"/>
+      <c r="U10" s="48"/>
+      <c r="V10" s="48"/>
+      <c r="W10" s="48"/>
     </row>
     <row r="11" ht="114.75" customHeight="1" spans="1:23">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="26"/>
-      <c r="K11" s="29"/>
-      <c r="L11" s="29"/>
-      <c r="M11" s="29"/>
-      <c r="N11" s="47"/>
-      <c r="O11" s="48"/>
-      <c r="P11" s="49"/>
-      <c r="Q11" s="26"/>
-      <c r="R11" s="26"/>
-      <c r="S11" s="26"/>
-      <c r="T11" s="46"/>
-      <c r="U11" s="46"/>
-      <c r="V11" s="46"/>
-      <c r="W11" s="46"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="31"/>
+      <c r="L11" s="31"/>
+      <c r="M11" s="31"/>
+      <c r="N11" s="49"/>
+      <c r="O11" s="50"/>
+      <c r="P11" s="51"/>
+      <c r="Q11" s="28"/>
+      <c r="R11" s="28"/>
+      <c r="S11" s="28"/>
+      <c r="T11" s="48"/>
+      <c r="U11" s="48"/>
+      <c r="V11" s="48"/>
+      <c r="W11" s="48"/>
     </row>
     <row r="12" ht="128.25" customHeight="1" spans="1:23">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="26"/>
-      <c r="K12" s="29"/>
-      <c r="L12" s="29"/>
-      <c r="M12" s="29"/>
-      <c r="N12" s="47"/>
-      <c r="O12" s="48"/>
-      <c r="P12" s="49"/>
-      <c r="Q12" s="26"/>
-      <c r="R12" s="26"/>
-      <c r="S12" s="26"/>
-      <c r="T12" s="46"/>
-      <c r="U12" s="46"/>
-      <c r="V12" s="46"/>
-      <c r="W12" s="46"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="28"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="31"/>
+      <c r="M12" s="31"/>
+      <c r="N12" s="49"/>
+      <c r="O12" s="50"/>
+      <c r="P12" s="51"/>
+      <c r="Q12" s="28"/>
+      <c r="R12" s="28"/>
+      <c r="S12" s="28"/>
+      <c r="T12" s="48"/>
+      <c r="U12" s="48"/>
+      <c r="V12" s="48"/>
+      <c r="W12" s="48"/>
     </row>
     <row r="13" customHeight="1" spans="1:23">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
-      <c r="J13" s="26"/>
-      <c r="K13" s="29"/>
-      <c r="L13" s="29"/>
-      <c r="M13" s="29"/>
-      <c r="N13" s="47"/>
-      <c r="O13" s="48"/>
-      <c r="P13" s="49"/>
-      <c r="Q13" s="26"/>
-      <c r="R13" s="26"/>
-      <c r="S13" s="26"/>
-      <c r="T13" s="46"/>
-      <c r="U13" s="46"/>
-      <c r="V13" s="46"/>
-      <c r="W13" s="46"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="28"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="31"/>
+      <c r="M13" s="31"/>
+      <c r="N13" s="49"/>
+      <c r="O13" s="50"/>
+      <c r="P13" s="51"/>
+      <c r="Q13" s="28"/>
+      <c r="R13" s="28"/>
+      <c r="S13" s="28"/>
+      <c r="T13" s="48"/>
+      <c r="U13" s="48"/>
+      <c r="V13" s="48"/>
+      <c r="W13" s="48"/>
     </row>
     <row r="14" customHeight="1" spans="1:23">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="26"/>
-      <c r="K14" s="29"/>
-      <c r="L14" s="29"/>
-      <c r="M14" s="29"/>
-      <c r="N14" s="47"/>
-      <c r="O14" s="48"/>
-      <c r="P14" s="49"/>
-      <c r="Q14" s="26"/>
-      <c r="R14" s="26"/>
-      <c r="S14" s="26"/>
-      <c r="T14" s="46"/>
-      <c r="U14" s="46"/>
-      <c r="V14" s="46"/>
-      <c r="W14" s="46"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
+      <c r="J14" s="28"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="31"/>
+      <c r="M14" s="31"/>
+      <c r="N14" s="49"/>
+      <c r="O14" s="50"/>
+      <c r="P14" s="51"/>
+      <c r="Q14" s="28"/>
+      <c r="R14" s="28"/>
+      <c r="S14" s="28"/>
+      <c r="T14" s="48"/>
+      <c r="U14" s="48"/>
+      <c r="V14" s="48"/>
+      <c r="W14" s="48"/>
     </row>
     <row r="15" customHeight="1" spans="1:23">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="26"/>
-      <c r="J15" s="26"/>
-      <c r="K15" s="29"/>
-      <c r="L15" s="29"/>
-      <c r="M15" s="29"/>
-      <c r="N15" s="47"/>
-      <c r="O15" s="48"/>
-      <c r="P15" s="49"/>
-      <c r="Q15" s="26"/>
-      <c r="R15" s="26"/>
-      <c r="S15" s="26"/>
-      <c r="T15" s="46"/>
-      <c r="U15" s="46"/>
-      <c r="V15" s="46"/>
-      <c r="W15" s="46"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="28"/>
+      <c r="K15" s="31"/>
+      <c r="L15" s="31"/>
+      <c r="M15" s="31"/>
+      <c r="N15" s="49"/>
+      <c r="O15" s="50"/>
+      <c r="P15" s="51"/>
+      <c r="Q15" s="28"/>
+      <c r="R15" s="28"/>
+      <c r="S15" s="28"/>
+      <c r="T15" s="48"/>
+      <c r="U15" s="48"/>
+      <c r="V15" s="48"/>
+      <c r="W15" s="48"/>
     </row>
     <row r="16" ht="86.25" customHeight="1" spans="1:23">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="26"/>
-      <c r="J16" s="26"/>
-      <c r="K16" s="29"/>
-      <c r="L16" s="29"/>
-      <c r="M16" s="29"/>
-      <c r="N16" s="50"/>
-      <c r="O16" s="51"/>
-      <c r="P16" s="52"/>
-      <c r="Q16" s="26"/>
-      <c r="R16" s="26"/>
-      <c r="S16" s="26"/>
-      <c r="T16" s="46"/>
-      <c r="U16" s="46"/>
-      <c r="V16" s="46"/>
-      <c r="W16" s="46"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="28"/>
+      <c r="K16" s="31"/>
+      <c r="L16" s="31"/>
+      <c r="M16" s="31"/>
+      <c r="N16" s="52"/>
+      <c r="O16" s="53"/>
+      <c r="P16" s="54"/>
+      <c r="Q16" s="28"/>
+      <c r="R16" s="28"/>
+      <c r="S16" s="28"/>
+      <c r="T16" s="48"/>
+      <c r="U16" s="48"/>
+      <c r="V16" s="48"/>
+      <c r="W16" s="48"/>
     </row>
     <row r="17" ht="93.75" customHeight="1" spans="1:23">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
-      <c r="C17" s="35" t="s">
+      <c r="C17" s="37" t="s">
         <v>62</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
-      <c r="H17" s="36" t="s">
+      <c r="H17" s="38" t="s">
         <v>67</v>
       </c>
-      <c r="I17" s="36"/>
-      <c r="J17" s="36"/>
-      <c r="K17" s="36" t="s">
+      <c r="I17" s="38"/>
+      <c r="J17" s="38"/>
+      <c r="K17" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="L17" s="36"/>
-      <c r="M17" s="36"/>
+      <c r="L17" s="38"/>
+      <c r="M17" s="38"/>
       <c r="N17" s="4">
         <v>400</v>
       </c>
       <c r="O17" s="4"/>
       <c r="P17" s="4"/>
-      <c r="Q17" s="36" t="s">
+      <c r="Q17" s="38" t="s">
         <v>60</v>
       </c>
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
-      <c r="T17" s="41" t="s">
+      <c r="T17" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="U17" s="42"/>
-      <c r="V17" s="42"/>
-      <c r="W17" s="42"/>
+      <c r="U17" s="44"/>
+      <c r="V17" s="44"/>
+      <c r="W17" s="44"/>
     </row>
     <row r="18" ht="150.75" customHeight="1" spans="1:23">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
-      <c r="C18" s="35" t="s">
+      <c r="C18" s="37" t="s">
         <v>62</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
-      <c r="H18" s="36" t="s">
+      <c r="H18" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="I18" s="36"/>
-      <c r="J18" s="36"/>
-      <c r="K18" s="36" t="s">
+      <c r="I18" s="38"/>
+      <c r="J18" s="38"/>
+      <c r="K18" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="L18" s="36"/>
-      <c r="M18" s="36"/>
+      <c r="L18" s="38"/>
+      <c r="M18" s="38"/>
       <c r="N18" s="4">
         <v>400</v>
       </c>
       <c r="O18" s="4"/>
       <c r="P18" s="4"/>
-      <c r="Q18" s="36" t="s">
+      <c r="Q18" s="38" t="s">
         <v>57</v>
       </c>
       <c r="R18" s="4"/>
       <c r="S18" s="4"/>
-      <c r="T18" s="41" t="s">
+      <c r="T18" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="U18" s="42"/>
-      <c r="V18" s="42"/>
-      <c r="W18" s="42"/>
+      <c r="U18" s="44"/>
+      <c r="V18" s="44"/>
+      <c r="W18" s="44"/>
     </row>
     <row r="19" ht="66.75" customHeight="1" spans="1:23">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
-      <c r="C19" s="53" t="s">
+      <c r="C19" s="55" t="s">
         <v>62</v>
       </c>
-      <c r="D19" s="54"/>
-      <c r="E19" s="54"/>
-      <c r="F19" s="54"/>
-      <c r="G19" s="54"/>
-      <c r="H19" s="55" t="s">
+      <c r="D19" s="56"/>
+      <c r="E19" s="56"/>
+      <c r="F19" s="56"/>
+      <c r="G19" s="56"/>
+      <c r="H19" s="57" t="s">
         <v>71</v>
       </c>
-      <c r="I19" s="55"/>
-      <c r="J19" s="55"/>
-      <c r="K19" s="55" t="s">
+      <c r="I19" s="57"/>
+      <c r="J19" s="57"/>
+      <c r="K19" s="57" t="s">
         <v>72</v>
       </c>
-      <c r="L19" s="55"/>
-      <c r="M19" s="55"/>
-      <c r="N19" s="54">
+      <c r="L19" s="57"/>
+      <c r="M19" s="57"/>
+      <c r="N19" s="56">
         <v>200</v>
       </c>
-      <c r="O19" s="54"/>
-      <c r="P19" s="54"/>
-      <c r="Q19" s="55" t="s">
+      <c r="O19" s="56"/>
+      <c r="P19" s="56"/>
+      <c r="Q19" s="57" t="s">
         <v>73</v>
       </c>
-      <c r="R19" s="54"/>
-      <c r="S19" s="54"/>
-      <c r="T19" s="56"/>
-      <c r="U19" s="57"/>
-      <c r="V19" s="57"/>
-      <c r="W19" s="57"/>
+      <c r="R19" s="56"/>
+      <c r="S19" s="56"/>
+      <c r="T19" s="58"/>
+      <c r="U19" s="59"/>
+      <c r="V19" s="59"/>
+      <c r="W19" s="59"/>
     </row>
     <row r="20" ht="129" customHeight="1" spans="1:23">
       <c r="A20" s="4" t="s">
         <v>74</v>
       </c>
       <c r="B20" s="4"/>
-      <c r="C20" s="58" t="s">
+      <c r="C20" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="59" t="s">
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="I20" s="60"/>
-      <c r="J20" s="61"/>
-      <c r="K20" s="30" t="s">
+      <c r="I20" s="62"/>
+      <c r="J20" s="63"/>
+      <c r="K20" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="L20" s="62"/>
-      <c r="M20" s="63"/>
-      <c r="N20" s="26">
+      <c r="L20" s="64"/>
+      <c r="M20" s="65"/>
+      <c r="N20" s="28">
         <v>200</v>
       </c>
-      <c r="O20" s="26"/>
-      <c r="P20" s="26"/>
-      <c r="Q20" s="26" t="s">
+      <c r="O20" s="28"/>
+      <c r="P20" s="28"/>
+      <c r="Q20" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="R20" s="26"/>
-      <c r="S20" s="26"/>
-      <c r="T20" s="46" t="s">
+      <c r="R20" s="28"/>
+      <c r="S20" s="28"/>
+      <c r="T20" s="48" t="s">
         <v>78</v>
       </c>
-      <c r="U20" s="46"/>
-      <c r="V20" s="46"/>
-      <c r="W20" s="46"/>
+      <c r="U20" s="48"/>
+      <c r="V20" s="48"/>
+      <c r="W20" s="48"/>
     </row>
     <row r="21" ht="102" customHeight="1" spans="1:23">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="B21" s="24"/>
-      <c r="C21" s="58" t="s">
+      <c r="B21" s="26"/>
+      <c r="C21" s="60" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="59" t="s">
+      <c r="D21" s="28"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="28"/>
+      <c r="H21" s="61" t="s">
         <v>79</v>
       </c>
-      <c r="I21" s="60"/>
-      <c r="J21" s="61"/>
-      <c r="K21" s="29" t="s">
+      <c r="I21" s="62"/>
+      <c r="J21" s="63"/>
+      <c r="K21" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="L21" s="29"/>
-      <c r="M21" s="29"/>
-      <c r="N21" s="26">
+      <c r="L21" s="31"/>
+      <c r="M21" s="31"/>
+      <c r="N21" s="28">
         <v>200</v>
       </c>
-      <c r="O21" s="26"/>
-      <c r="P21" s="26"/>
-      <c r="Q21" s="26" t="s">
+      <c r="O21" s="28"/>
+      <c r="P21" s="28"/>
+      <c r="Q21" s="28" t="s">
         <v>81</v>
       </c>
-      <c r="R21" s="26"/>
-      <c r="S21" s="26"/>
-      <c r="T21" s="46" t="s">
+      <c r="R21" s="28"/>
+      <c r="S21" s="28"/>
+      <c r="T21" s="48" t="s">
         <v>82</v>
       </c>
-      <c r="U21" s="46"/>
-      <c r="V21" s="46"/>
-      <c r="W21" s="46"/>
+      <c r="U21" s="48"/>
+      <c r="V21" s="48"/>
+      <c r="W21" s="48"/>
     </row>
     <row r="22" ht="185.25" customHeight="1" spans="1:23">
-      <c r="A22" s="64"/>
-      <c r="B22" s="65"/>
-      <c r="C22" s="66" t="s">
+      <c r="A22" s="66"/>
+      <c r="B22" s="67"/>
+      <c r="C22" s="68" t="s">
         <v>62</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
-      <c r="H22" s="67" t="s">
+      <c r="H22" s="69" t="s">
         <v>83</v>
       </c>
-      <c r="I22" s="68"/>
-      <c r="J22" s="69"/>
-      <c r="K22" s="36" t="s">
+      <c r="I22" s="70"/>
+      <c r="J22" s="71"/>
+      <c r="K22" s="38" t="s">
         <v>84</v>
       </c>
-      <c r="L22" s="36"/>
-      <c r="M22" s="36"/>
+      <c r="L22" s="38"/>
+      <c r="M22" s="38"/>
       <c r="N22" s="4">
         <v>400</v>
       </c>
       <c r="O22" s="4"/>
       <c r="P22" s="4"/>
-      <c r="Q22" s="70" t="s">
+      <c r="Q22" s="72" t="s">
         <v>85</v>
       </c>
-      <c r="R22" s="71"/>
-      <c r="S22" s="72"/>
-      <c r="T22" s="37" t="s">
+      <c r="R22" s="73"/>
+      <c r="S22" s="74"/>
+      <c r="T22" s="39" t="s">
         <v>86</v>
       </c>
-      <c r="U22" s="37"/>
-      <c r="V22" s="37"/>
-      <c r="W22" s="37"/>
+      <c r="U22" s="39"/>
+      <c r="V22" s="39"/>
+      <c r="W22" s="39"/>
     </row>
     <row r="23" ht="145.5" customHeight="1" spans="1:23">
       <c r="A23" s="4" t="s">
         <v>87</v>
       </c>
       <c r="B23" s="4"/>
-      <c r="C23" s="25" t="s">
+      <c r="C23" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="29" t="s">
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="31" t="s">
         <v>88</v>
       </c>
-      <c r="I23" s="29"/>
-      <c r="J23" s="29"/>
-      <c r="K23" s="29" t="s">
+      <c r="I23" s="31"/>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="L23" s="29"/>
-      <c r="M23" s="29"/>
-      <c r="N23" s="26">
+      <c r="L23" s="31"/>
+      <c r="M23" s="31"/>
+      <c r="N23" s="28">
         <v>200</v>
       </c>
-      <c r="O23" s="26"/>
-      <c r="P23" s="26"/>
-      <c r="Q23" s="26" t="s">
+      <c r="O23" s="28"/>
+      <c r="P23" s="28"/>
+      <c r="Q23" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="R23" s="26"/>
-      <c r="S23" s="26"/>
-      <c r="T23" s="46" t="s">
+      <c r="R23" s="28"/>
+      <c r="S23" s="28"/>
+      <c r="T23" s="48" t="s">
         <v>91</v>
       </c>
-      <c r="U23" s="73"/>
-      <c r="V23" s="73"/>
-      <c r="W23" s="73"/>
+      <c r="U23" s="75"/>
+      <c r="V23" s="75"/>
+      <c r="W23" s="75"/>
     </row>
     <row r="24" ht="238.5" customHeight="1" spans="1:23">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
-      <c r="C24" s="35" t="s">
+      <c r="C24" s="37" t="s">
         <v>62</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
-      <c r="H24" s="37" t="s">
+      <c r="H24" s="39" t="s">
         <v>92</v>
       </c>
-      <c r="I24" s="37"/>
-      <c r="J24" s="37"/>
-      <c r="K24" s="36" t="s">
+      <c r="I24" s="39"/>
+      <c r="J24" s="39"/>
+      <c r="K24" s="38" t="s">
         <v>93</v>
       </c>
-      <c r="L24" s="36"/>
-      <c r="M24" s="36"/>
+      <c r="L24" s="38"/>
+      <c r="M24" s="38"/>
       <c r="N24" s="4">
         <v>400</v>
       </c>
       <c r="O24" s="4"/>
       <c r="P24" s="4"/>
-      <c r="Q24" s="70" t="s">
+      <c r="Q24" s="72" t="s">
         <v>94</v>
       </c>
-      <c r="R24" s="71"/>
-      <c r="S24" s="72"/>
-      <c r="T24" s="37" t="s">
+      <c r="R24" s="73"/>
+      <c r="S24" s="74"/>
+      <c r="T24" s="39" t="s">
         <v>86</v>
       </c>
-      <c r="U24" s="37"/>
-      <c r="V24" s="37"/>
-      <c r="W24" s="37"/>
+      <c r="U24" s="39"/>
+      <c r="V24" s="39"/>
+      <c r="W24" s="39"/>
     </row>
     <row r="25" spans="1:23">
-      <c r="A25" s="15" t="s">
+      <c r="A25" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="16"/>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="16"/>
-      <c r="O25" s="16"/>
-      <c r="P25" s="16"/>
-      <c r="Q25" s="16"/>
-      <c r="R25" s="16"/>
-      <c r="S25" s="16"/>
-      <c r="T25" s="16"/>
-      <c r="U25" s="16"/>
-      <c r="V25" s="16"/>
-      <c r="W25" s="17"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
+      <c r="J25" s="18"/>
+      <c r="K25" s="18"/>
+      <c r="L25" s="18"/>
+      <c r="M25" s="18"/>
+      <c r="N25" s="18"/>
+      <c r="O25" s="18"/>
+      <c r="P25" s="18"/>
+      <c r="Q25" s="18"/>
+      <c r="R25" s="18"/>
+      <c r="S25" s="18"/>
+      <c r="T25" s="18"/>
+      <c r="U25" s="18"/>
+      <c r="V25" s="18"/>
+      <c r="W25" s="19"/>
     </row>
     <row r="26" ht="109.5" customHeight="1" spans="1:23">
-      <c r="A26" s="74" t="s">
+      <c r="A26" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="75"/>
-      <c r="C26" s="26" t="s">
+      <c r="B26" s="77"/>
+      <c r="C26" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="D26" s="26"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="26"/>
-      <c r="H26" s="27" t="s">
+      <c r="D26" s="28"/>
+      <c r="E26" s="28"/>
+      <c r="F26" s="28"/>
+      <c r="G26" s="28"/>
+      <c r="H26" s="29" t="s">
         <v>97</v>
       </c>
-      <c r="I26" s="28"/>
-      <c r="J26" s="25"/>
-      <c r="K26" s="29" t="s">
+      <c r="I26" s="30"/>
+      <c r="J26" s="27"/>
+      <c r="K26" s="31" t="s">
         <v>98</v>
       </c>
-      <c r="L26" s="29"/>
-      <c r="M26" s="29"/>
-      <c r="N26" s="26">
+      <c r="L26" s="31"/>
+      <c r="M26" s="31"/>
+      <c r="N26" s="28">
         <v>201</v>
       </c>
-      <c r="O26" s="26"/>
-      <c r="P26" s="26"/>
-      <c r="Q26" s="26" t="s">
+      <c r="O26" s="28"/>
+      <c r="P26" s="28"/>
+      <c r="Q26" s="28" t="s">
         <v>99</v>
       </c>
-      <c r="R26" s="26"/>
-      <c r="S26" s="26"/>
-      <c r="T26" s="30" t="s">
+      <c r="R26" s="28"/>
+      <c r="S26" s="28"/>
+      <c r="T26" s="32" t="s">
         <v>100</v>
       </c>
-      <c r="U26" s="31"/>
-      <c r="V26" s="31"/>
-      <c r="W26" s="32"/>
+      <c r="U26" s="33"/>
+      <c r="V26" s="33"/>
+      <c r="W26" s="34"/>
     </row>
     <row r="27" ht="152.25" customHeight="1" spans="1:23">
-      <c r="A27" s="76"/>
-      <c r="B27" s="77"/>
-      <c r="C27" s="78" t="s">
+      <c r="A27" s="78"/>
+      <c r="B27" s="79"/>
+      <c r="C27" s="80" t="s">
         <v>96</v>
       </c>
-      <c r="D27" s="78"/>
-      <c r="E27" s="78"/>
-      <c r="F27" s="78"/>
-      <c r="G27" s="78"/>
-      <c r="H27" s="67" t="s">
+      <c r="D27" s="80"/>
+      <c r="E27" s="80"/>
+      <c r="F27" s="80"/>
+      <c r="G27" s="80"/>
+      <c r="H27" s="69" t="s">
         <v>101</v>
       </c>
-      <c r="I27" s="68"/>
-      <c r="J27" s="69"/>
-      <c r="K27" s="67" t="s">
+      <c r="I27" s="70"/>
+      <c r="J27" s="71"/>
+      <c r="K27" s="69" t="s">
         <v>102</v>
       </c>
-      <c r="L27" s="68"/>
-      <c r="M27" s="69"/>
-      <c r="N27" s="79">
+      <c r="L27" s="70"/>
+      <c r="M27" s="71"/>
+      <c r="N27" s="81">
         <v>400</v>
       </c>
-      <c r="O27" s="80"/>
-      <c r="P27" s="35"/>
-      <c r="Q27" s="67" t="s">
+      <c r="O27" s="82"/>
+      <c r="P27" s="37"/>
+      <c r="Q27" s="69" t="s">
         <v>103</v>
       </c>
-      <c r="R27" s="80"/>
-      <c r="S27" s="35"/>
-      <c r="T27" s="41" t="s">
+      <c r="R27" s="82"/>
+      <c r="S27" s="37"/>
+      <c r="T27" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="U27" s="42"/>
-      <c r="V27" s="42"/>
-      <c r="W27" s="42"/>
+      <c r="U27" s="44"/>
+      <c r="V27" s="44"/>
+      <c r="W27" s="44"/>
     </row>
     <row r="28" ht="353.25" customHeight="1" spans="1:23">
-      <c r="A28" s="76"/>
-      <c r="B28" s="77"/>
-      <c r="C28" s="78" t="s">
+      <c r="A28" s="78"/>
+      <c r="B28" s="79"/>
+      <c r="C28" s="80" t="s">
         <v>96</v>
       </c>
-      <c r="D28" s="78"/>
-      <c r="E28" s="78"/>
-      <c r="F28" s="78"/>
-      <c r="G28" s="78"/>
-      <c r="H28" s="67" t="s">
+      <c r="D28" s="80"/>
+      <c r="E28" s="80"/>
+      <c r="F28" s="80"/>
+      <c r="G28" s="80"/>
+      <c r="H28" s="69" t="s">
         <v>104</v>
       </c>
-      <c r="I28" s="68"/>
-      <c r="J28" s="69"/>
-      <c r="K28" s="67" t="s">
+      <c r="I28" s="70"/>
+      <c r="J28" s="71"/>
+      <c r="K28" s="69" t="s">
         <v>105</v>
       </c>
-      <c r="L28" s="68"/>
-      <c r="M28" s="69"/>
-      <c r="N28" s="79">
+      <c r="L28" s="70"/>
+      <c r="M28" s="71"/>
+      <c r="N28" s="81">
         <v>400</v>
       </c>
-      <c r="O28" s="80"/>
-      <c r="P28" s="35"/>
-      <c r="Q28" s="67" t="s">
+      <c r="O28" s="82"/>
+      <c r="P28" s="37"/>
+      <c r="Q28" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="R28" s="68"/>
-      <c r="S28" s="69"/>
-      <c r="T28" s="41" t="s">
+      <c r="R28" s="70"/>
+      <c r="S28" s="71"/>
+      <c r="T28" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="U28" s="42"/>
-      <c r="V28" s="42"/>
-      <c r="W28" s="42"/>
+      <c r="U28" s="44"/>
+      <c r="V28" s="44"/>
+      <c r="W28" s="44"/>
     </row>
     <row r="29" ht="285" customHeight="1" spans="1:23">
-      <c r="A29" s="81"/>
-      <c r="B29" s="82"/>
-      <c r="C29" s="78" t="s">
+      <c r="A29" s="83"/>
+      <c r="B29" s="84"/>
+      <c r="C29" s="80" t="s">
         <v>96</v>
       </c>
-      <c r="D29" s="78"/>
-      <c r="E29" s="78"/>
-      <c r="F29" s="78"/>
-      <c r="G29" s="78"/>
-      <c r="H29" s="67" t="s">
+      <c r="D29" s="80"/>
+      <c r="E29" s="80"/>
+      <c r="F29" s="80"/>
+      <c r="G29" s="80"/>
+      <c r="H29" s="69" t="s">
         <v>107</v>
       </c>
-      <c r="I29" s="68"/>
-      <c r="J29" s="69"/>
-      <c r="K29" s="67" t="s">
+      <c r="I29" s="70"/>
+      <c r="J29" s="71"/>
+      <c r="K29" s="69" t="s">
         <v>108</v>
       </c>
-      <c r="L29" s="68"/>
-      <c r="M29" s="69"/>
-      <c r="N29" s="79">
+      <c r="L29" s="70"/>
+      <c r="M29" s="71"/>
+      <c r="N29" s="81">
         <v>400</v>
       </c>
-      <c r="O29" s="80"/>
-      <c r="P29" s="35"/>
-      <c r="Q29" s="67" t="s">
+      <c r="O29" s="82"/>
+      <c r="P29" s="37"/>
+      <c r="Q29" s="69" t="s">
         <v>109</v>
       </c>
-      <c r="R29" s="68"/>
-      <c r="S29" s="69"/>
-      <c r="T29" s="41" t="s">
+      <c r="R29" s="70"/>
+      <c r="S29" s="71"/>
+      <c r="T29" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="U29" s="42"/>
-      <c r="V29" s="42"/>
-      <c r="W29" s="42"/>
+      <c r="U29" s="44"/>
+      <c r="V29" s="44"/>
+      <c r="W29" s="44"/>
     </row>
     <row r="30" ht="98.25" customHeight="1" spans="1:23">
-      <c r="A30" s="83" t="s">
+      <c r="A30" s="85" t="s">
         <v>74</v>
       </c>
-      <c r="B30" s="24"/>
-      <c r="C30" s="78" t="s">
+      <c r="B30" s="26"/>
+      <c r="C30" s="80" t="s">
         <v>96</v>
       </c>
-      <c r="D30" s="78"/>
-      <c r="E30" s="78"/>
-      <c r="F30" s="78"/>
-      <c r="G30" s="78"/>
-      <c r="H30" s="59" t="s">
+      <c r="D30" s="80"/>
+      <c r="E30" s="80"/>
+      <c r="F30" s="80"/>
+      <c r="G30" s="80"/>
+      <c r="H30" s="61" t="s">
         <v>110</v>
       </c>
-      <c r="I30" s="60"/>
-      <c r="J30" s="61"/>
-      <c r="K30" s="30" t="s">
+      <c r="I30" s="62"/>
+      <c r="J30" s="63"/>
+      <c r="K30" s="32" t="s">
         <v>111</v>
       </c>
-      <c r="L30" s="62"/>
-      <c r="M30" s="63"/>
-      <c r="N30" s="27">
+      <c r="L30" s="64"/>
+      <c r="M30" s="65"/>
+      <c r="N30" s="29">
         <v>200</v>
       </c>
-      <c r="O30" s="28"/>
-      <c r="P30" s="25"/>
-      <c r="Q30" s="26" t="s">
+      <c r="O30" s="30"/>
+      <c r="P30" s="27"/>
+      <c r="Q30" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="R30" s="26"/>
-      <c r="S30" s="26"/>
-      <c r="T30" s="46" t="s">
+      <c r="R30" s="28"/>
+      <c r="S30" s="28"/>
+      <c r="T30" s="48" t="s">
         <v>78</v>
       </c>
-      <c r="U30" s="46"/>
-      <c r="V30" s="46"/>
-      <c r="W30" s="46"/>
+      <c r="U30" s="48"/>
+      <c r="V30" s="48"/>
+      <c r="W30" s="48"/>
     </row>
     <row r="31" ht="82.5" customHeight="1" spans="1:23">
       <c r="A31" s="4" t="s">
         <v>74</v>
       </c>
       <c r="B31" s="4"/>
-      <c r="C31" s="78" t="s">
+      <c r="C31" s="80" t="s">
         <v>112</v>
       </c>
-      <c r="D31" s="78"/>
-      <c r="E31" s="78"/>
-      <c r="F31" s="78"/>
-      <c r="G31" s="78"/>
-      <c r="H31" s="59" t="s">
+      <c r="D31" s="80"/>
+      <c r="E31" s="80"/>
+      <c r="F31" s="80"/>
+      <c r="G31" s="80"/>
+      <c r="H31" s="61" t="s">
         <v>113</v>
       </c>
-      <c r="I31" s="60"/>
-      <c r="J31" s="61"/>
-      <c r="K31" s="29" t="s">
+      <c r="I31" s="62"/>
+      <c r="J31" s="63"/>
+      <c r="K31" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="L31" s="29"/>
-      <c r="M31" s="29"/>
-      <c r="N31" s="27">
+      <c r="L31" s="31"/>
+      <c r="M31" s="31"/>
+      <c r="N31" s="29">
         <v>200</v>
       </c>
-      <c r="O31" s="28"/>
-      <c r="P31" s="25"/>
-      <c r="Q31" s="26" t="s">
+      <c r="O31" s="30"/>
+      <c r="P31" s="27"/>
+      <c r="Q31" s="28" t="s">
         <v>115</v>
       </c>
-      <c r="R31" s="26"/>
-      <c r="S31" s="26"/>
-      <c r="T31" s="46" t="s">
+      <c r="R31" s="28"/>
+      <c r="S31" s="28"/>
+      <c r="T31" s="48" t="s">
         <v>116</v>
       </c>
-      <c r="U31" s="46"/>
-      <c r="V31" s="46"/>
-      <c r="W31" s="46"/>
+      <c r="U31" s="48"/>
+      <c r="V31" s="48"/>
+      <c r="W31" s="48"/>
     </row>
     <row r="32" ht="225.75" customHeight="1" spans="1:23">
       <c r="A32" s="4"/>
       <c r="B32" s="4"/>
-      <c r="C32" s="78" t="s">
+      <c r="C32" s="80" t="s">
         <v>112</v>
       </c>
-      <c r="D32" s="78"/>
-      <c r="E32" s="78"/>
-      <c r="F32" s="78"/>
-      <c r="G32" s="78"/>
-      <c r="H32" s="67" t="s">
+      <c r="D32" s="80"/>
+      <c r="E32" s="80"/>
+      <c r="F32" s="80"/>
+      <c r="G32" s="80"/>
+      <c r="H32" s="69" t="s">
         <v>117</v>
       </c>
-      <c r="I32" s="68"/>
-      <c r="J32" s="69"/>
-      <c r="K32" s="36" t="s">
+      <c r="I32" s="70"/>
+      <c r="J32" s="71"/>
+      <c r="K32" s="38" t="s">
         <v>118</v>
       </c>
-      <c r="L32" s="36"/>
-      <c r="M32" s="36"/>
-      <c r="N32" s="79">
+      <c r="L32" s="38"/>
+      <c r="M32" s="38"/>
+      <c r="N32" s="81">
         <v>400</v>
       </c>
-      <c r="O32" s="80"/>
-      <c r="P32" s="35"/>
-      <c r="Q32" s="39" t="s">
+      <c r="O32" s="82"/>
+      <c r="P32" s="37"/>
+      <c r="Q32" s="41" t="s">
         <v>119</v>
       </c>
-      <c r="R32" s="40"/>
-      <c r="S32" s="40"/>
-      <c r="T32" s="37" t="s">
+      <c r="R32" s="42"/>
+      <c r="S32" s="42"/>
+      <c r="T32" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="U32" s="37"/>
-      <c r="V32" s="37"/>
-      <c r="W32" s="37"/>
+      <c r="U32" s="39"/>
+      <c r="V32" s="39"/>
+      <c r="W32" s="39"/>
     </row>
     <row r="33" ht="120" customHeight="1" spans="1:25">
       <c r="A33" s="4" t="s">
         <v>121</v>
       </c>
       <c r="B33" s="4"/>
-      <c r="C33" s="78" t="s">
+      <c r="C33" s="80" t="s">
         <v>112</v>
       </c>
-      <c r="D33" s="78"/>
-      <c r="E33" s="78"/>
-      <c r="F33" s="78"/>
-      <c r="G33" s="78"/>
-      <c r="H33" s="29" t="s">
+      <c r="D33" s="80"/>
+      <c r="E33" s="80"/>
+      <c r="F33" s="80"/>
+      <c r="G33" s="80"/>
+      <c r="H33" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="I33" s="29"/>
-      <c r="J33" s="29"/>
-      <c r="K33" s="29" t="s">
+      <c r="I33" s="31"/>
+      <c r="J33" s="31"/>
+      <c r="K33" s="31" t="s">
         <v>123</v>
       </c>
-      <c r="L33" s="29"/>
-      <c r="M33" s="29"/>
-      <c r="N33" s="26">
+      <c r="L33" s="31"/>
+      <c r="M33" s="31"/>
+      <c r="N33" s="28">
         <v>200</v>
       </c>
-      <c r="O33" s="26"/>
-      <c r="P33" s="26"/>
-      <c r="Q33" s="26" t="s">
+      <c r="O33" s="28"/>
+      <c r="P33" s="28"/>
+      <c r="Q33" s="28" t="s">
         <v>124</v>
       </c>
-      <c r="R33" s="26"/>
-      <c r="S33" s="26"/>
-      <c r="T33" s="46" t="s">
+      <c r="R33" s="28"/>
+      <c r="S33" s="28"/>
+      <c r="T33" s="48" t="s">
         <v>125</v>
       </c>
-      <c r="U33" s="46"/>
-      <c r="V33" s="46"/>
-      <c r="W33" s="46"/>
+      <c r="U33" s="48"/>
+      <c r="V33" s="48"/>
+      <c r="W33" s="48"/>
     </row>
     <row r="34" ht="116.25" customHeight="1" spans="1:25">
       <c r="A34" s="4"/>
       <c r="B34" s="4"/>
-      <c r="C34" s="55" t="s">
+      <c r="C34" s="57" t="s">
         <v>112</v>
       </c>
-      <c r="D34" s="55"/>
-      <c r="E34" s="55"/>
-      <c r="F34" s="55"/>
-      <c r="G34" s="55"/>
-      <c r="H34" s="55" t="s">
+      <c r="D34" s="57"/>
+      <c r="E34" s="57"/>
+      <c r="F34" s="57"/>
+      <c r="G34" s="57"/>
+      <c r="H34" s="57" t="s">
         <v>126</v>
       </c>
-      <c r="I34" s="55"/>
-      <c r="J34" s="55"/>
-      <c r="K34" s="55" t="s">
+      <c r="I34" s="57"/>
+      <c r="J34" s="57"/>
+      <c r="K34" s="57" t="s">
         <v>127</v>
       </c>
-      <c r="L34" s="55"/>
-      <c r="M34" s="55"/>
-      <c r="N34" s="54">
+      <c r="L34" s="57"/>
+      <c r="M34" s="57"/>
+      <c r="N34" s="56">
         <v>200</v>
       </c>
-      <c r="O34" s="54"/>
-      <c r="P34" s="54"/>
-      <c r="Q34" s="55" t="s">
+      <c r="O34" s="56"/>
+      <c r="P34" s="56"/>
+      <c r="Q34" s="57" t="s">
         <v>73</v>
       </c>
-      <c r="R34" s="54"/>
-      <c r="S34" s="54"/>
-      <c r="T34" s="56"/>
-      <c r="U34" s="57"/>
-      <c r="V34" s="57"/>
-      <c r="W34" s="57"/>
+      <c r="R34" s="56"/>
+      <c r="S34" s="56"/>
+      <c r="T34" s="58"/>
+      <c r="U34" s="59"/>
+      <c r="V34" s="59"/>
+      <c r="W34" s="59"/>
     </row>
     <row r="35" ht="180.75" customHeight="1" spans="1:25">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
-      <c r="C35" s="84" t="s">
+      <c r="C35" s="86" t="s">
         <v>112</v>
       </c>
-      <c r="D35" s="84"/>
-      <c r="E35" s="84"/>
-      <c r="F35" s="84"/>
-      <c r="G35" s="84"/>
-      <c r="H35" s="84" t="s">
+      <c r="D35" s="86"/>
+      <c r="E35" s="86"/>
+      <c r="F35" s="86"/>
+      <c r="G35" s="86"/>
+      <c r="H35" s="86" t="s">
         <v>128</v>
       </c>
-      <c r="I35" s="84"/>
-      <c r="J35" s="84"/>
-      <c r="K35" s="84" t="s">
+      <c r="I35" s="86"/>
+      <c r="J35" s="86"/>
+      <c r="K35" s="86" t="s">
         <v>129</v>
       </c>
-      <c r="L35" s="84"/>
-      <c r="M35" s="84"/>
-      <c r="N35" s="85">
+      <c r="L35" s="86"/>
+      <c r="M35" s="86"/>
+      <c r="N35" s="87">
         <v>400</v>
       </c>
-      <c r="O35" s="85"/>
-      <c r="P35" s="85"/>
-      <c r="Q35" s="84" t="s">
+      <c r="O35" s="87"/>
+      <c r="P35" s="87"/>
+      <c r="Q35" s="86" t="s">
         <v>130</v>
       </c>
-      <c r="R35" s="85"/>
-      <c r="S35" s="85"/>
-      <c r="T35" s="86" t="s">
+      <c r="R35" s="87"/>
+      <c r="S35" s="87"/>
+      <c r="T35" s="88" t="s">
         <v>48</v>
       </c>
-      <c r="U35" s="87"/>
-      <c r="V35" s="87"/>
-      <c r="W35" s="87"/>
+      <c r="U35" s="89"/>
+      <c r="V35" s="89"/>
+      <c r="W35" s="89"/>
     </row>
     <row r="36" ht="162.75" customHeight="1" spans="1:25">
       <c r="A36" s="4"/>
       <c r="B36" s="4"/>
-      <c r="C36" s="84" t="s">
+      <c r="C36" s="86" t="s">
         <v>112</v>
       </c>
-      <c r="D36" s="84"/>
-      <c r="E36" s="84"/>
-      <c r="F36" s="84"/>
-      <c r="G36" s="84"/>
-      <c r="H36" s="84" t="s">
+      <c r="D36" s="86"/>
+      <c r="E36" s="86"/>
+      <c r="F36" s="86"/>
+      <c r="G36" s="86"/>
+      <c r="H36" s="86" t="s">
         <v>131</v>
       </c>
-      <c r="I36" s="84"/>
-      <c r="J36" s="84"/>
-      <c r="K36" s="84" t="s">
+      <c r="I36" s="86"/>
+      <c r="J36" s="86"/>
+      <c r="K36" s="86" t="s">
         <v>132</v>
       </c>
-      <c r="L36" s="84"/>
-      <c r="M36" s="84"/>
-      <c r="N36" s="85">
+      <c r="L36" s="86"/>
+      <c r="M36" s="86"/>
+      <c r="N36" s="87">
         <v>400</v>
       </c>
-      <c r="O36" s="85"/>
-      <c r="P36" s="85"/>
-      <c r="Q36" s="84" t="s">
+      <c r="O36" s="87"/>
+      <c r="P36" s="87"/>
+      <c r="Q36" s="86" t="s">
         <v>133</v>
       </c>
-      <c r="R36" s="85"/>
-      <c r="S36" s="85"/>
-      <c r="T36" s="86" t="s">
+      <c r="R36" s="87"/>
+      <c r="S36" s="87"/>
+      <c r="T36" s="88" t="s">
         <v>48</v>
       </c>
-      <c r="U36" s="87"/>
-      <c r="V36" s="87"/>
-      <c r="W36" s="87"/>
+      <c r="U36" s="89"/>
+      <c r="V36" s="89"/>
+      <c r="W36" s="89"/>
     </row>
     <row r="37" ht="124.5" customHeight="1" spans="1:25">
-      <c r="A37" s="23" t="s">
+      <c r="A37" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="B37" s="83"/>
-      <c r="C37" s="88" t="s">
+      <c r="B37" s="85"/>
+      <c r="C37" s="90" t="s">
         <v>112</v>
       </c>
-      <c r="D37" s="88"/>
-      <c r="E37" s="88"/>
-      <c r="F37" s="88"/>
-      <c r="G37" s="88"/>
-      <c r="H37" s="29" t="s">
+      <c r="D37" s="90"/>
+      <c r="E37" s="90"/>
+      <c r="F37" s="90"/>
+      <c r="G37" s="90"/>
+      <c r="H37" s="31" t="s">
         <v>134</v>
       </c>
-      <c r="I37" s="29"/>
-      <c r="J37" s="29"/>
-      <c r="K37" s="29" t="s">
+      <c r="I37" s="31"/>
+      <c r="J37" s="31"/>
+      <c r="K37" s="31" t="s">
         <v>135</v>
       </c>
-      <c r="L37" s="29"/>
-      <c r="M37" s="29"/>
-      <c r="N37" s="26">
+      <c r="L37" s="31"/>
+      <c r="M37" s="31"/>
+      <c r="N37" s="28">
         <v>200</v>
       </c>
-      <c r="O37" s="26"/>
-      <c r="P37" s="26"/>
-      <c r="Q37" s="26" t="s">
+      <c r="O37" s="28"/>
+      <c r="P37" s="28"/>
+      <c r="Q37" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="R37" s="26"/>
-      <c r="S37" s="26"/>
-      <c r="T37" s="46" t="s">
+      <c r="R37" s="28"/>
+      <c r="S37" s="28"/>
+      <c r="T37" s="48" t="s">
         <v>91</v>
       </c>
-      <c r="U37" s="73"/>
-      <c r="V37" s="73"/>
-      <c r="W37" s="73"/>
+      <c r="U37" s="75"/>
+      <c r="V37" s="75"/>
+      <c r="W37" s="75"/>
     </row>
     <row r="38" ht="202.5" customHeight="1" spans="1:25">
-      <c r="A38" s="64"/>
-      <c r="B38" s="89"/>
-      <c r="C38" s="88" t="s">
+      <c r="A38" s="66"/>
+      <c r="B38" s="91"/>
+      <c r="C38" s="90" t="s">
         <v>112</v>
       </c>
-      <c r="D38" s="88"/>
-      <c r="E38" s="88"/>
-      <c r="F38" s="88"/>
-      <c r="G38" s="88"/>
-      <c r="H38" s="90" t="s">
+      <c r="D38" s="90"/>
+      <c r="E38" s="90"/>
+      <c r="F38" s="90"/>
+      <c r="G38" s="90"/>
+      <c r="H38" s="92" t="s">
         <v>136</v>
       </c>
-      <c r="I38" s="90"/>
-      <c r="J38" s="90"/>
-      <c r="K38" s="90" t="s">
+      <c r="I38" s="92"/>
+      <c r="J38" s="92"/>
+      <c r="K38" s="92" t="s">
         <v>137</v>
       </c>
-      <c r="L38" s="90"/>
-      <c r="M38" s="90"/>
-      <c r="N38" s="91">
+      <c r="L38" s="92"/>
+      <c r="M38" s="92"/>
+      <c r="N38" s="93">
         <v>400</v>
       </c>
-      <c r="O38" s="91"/>
-      <c r="P38" s="91"/>
-      <c r="Q38" s="39" t="s">
+      <c r="O38" s="93"/>
+      <c r="P38" s="93"/>
+      <c r="Q38" s="41" t="s">
         <v>138</v>
       </c>
-      <c r="R38" s="40"/>
-      <c r="S38" s="40"/>
-      <c r="T38" s="37" t="s">
+      <c r="R38" s="42"/>
+      <c r="S38" s="42"/>
+      <c r="T38" s="39" t="s">
         <v>116</v>
       </c>
-      <c r="U38" s="37"/>
-      <c r="V38" s="37"/>
-      <c r="W38" s="37"/>
+      <c r="U38" s="39"/>
+      <c r="V38" s="39"/>
+      <c r="W38" s="39"/>
     </row>
     <row r="39" spans="1:25">
-      <c r="A39" s="15" t="s">
+      <c r="A39" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="B39" s="16"/>
-      <c r="C39" s="16"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="16"/>
-      <c r="F39" s="16"/>
-      <c r="G39" s="16"/>
-      <c r="H39" s="16"/>
-      <c r="I39" s="16"/>
-      <c r="J39" s="16"/>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="16"/>
-      <c r="O39" s="16"/>
-      <c r="P39" s="16"/>
-      <c r="Q39" s="16"/>
-      <c r="R39" s="16"/>
-      <c r="S39" s="16"/>
-      <c r="T39" s="16"/>
-      <c r="U39" s="16"/>
-      <c r="V39" s="16"/>
-      <c r="W39" s="17"/>
+      <c r="B39" s="18"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="18"/>
+      <c r="G39" s="18"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="18"/>
+      <c r="J39" s="18"/>
+      <c r="K39" s="18"/>
+      <c r="L39" s="18"/>
+      <c r="M39" s="18"/>
+      <c r="N39" s="18"/>
+      <c r="O39" s="18"/>
+      <c r="P39" s="18"/>
+      <c r="Q39" s="18"/>
+      <c r="R39" s="18"/>
+      <c r="S39" s="18"/>
+      <c r="T39" s="18"/>
+      <c r="U39" s="18"/>
+      <c r="V39" s="18"/>
+      <c r="W39" s="19"/>
     </row>
     <row r="40" ht="102.75" customHeight="1" spans="1:25">
       <c r="A40" s="4" t="s">
         <v>39</v>
       </c>
       <c r="B40" s="4"/>
-      <c r="C40" s="92" t="s">
+      <c r="C40" s="94" t="s">
         <v>140</v>
       </c>
-      <c r="D40" s="92"/>
-      <c r="E40" s="92"/>
-      <c r="F40" s="92"/>
-      <c r="G40" s="92"/>
-      <c r="H40" s="27" t="s">
+      <c r="D40" s="94"/>
+      <c r="E40" s="94"/>
+      <c r="F40" s="94"/>
+      <c r="G40" s="94"/>
+      <c r="H40" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="I40" s="28"/>
-      <c r="J40" s="25"/>
-      <c r="K40" s="29" t="s">
+      <c r="I40" s="30"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="31" t="s">
         <v>142</v>
       </c>
-      <c r="L40" s="29"/>
-      <c r="M40" s="29"/>
-      <c r="N40" s="26">
+      <c r="L40" s="31"/>
+      <c r="M40" s="31"/>
+      <c r="N40" s="28">
         <v>201</v>
       </c>
-      <c r="O40" s="26"/>
-      <c r="P40" s="26"/>
-      <c r="Q40" s="26" t="s">
+      <c r="O40" s="28"/>
+      <c r="P40" s="28"/>
+      <c r="Q40" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="R40" s="26"/>
-      <c r="S40" s="26"/>
-      <c r="T40" s="30" t="s">
+      <c r="R40" s="28"/>
+      <c r="S40" s="28"/>
+      <c r="T40" s="32" t="s">
         <v>100</v>
       </c>
-      <c r="U40" s="31"/>
-      <c r="V40" s="31"/>
-      <c r="W40" s="32"/>
+      <c r="U40" s="33"/>
+      <c r="V40" s="33"/>
+      <c r="W40" s="34"/>
     </row>
     <row r="41" ht="134.25" customHeight="1" spans="1:25">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
-      <c r="C41" s="91" t="s">
+      <c r="C41" s="93" t="s">
         <v>140</v>
       </c>
-      <c r="D41" s="91"/>
-      <c r="E41" s="91"/>
-      <c r="F41" s="91"/>
-      <c r="G41" s="91"/>
-      <c r="H41" s="93" t="s">
+      <c r="D41" s="93"/>
+      <c r="E41" s="93"/>
+      <c r="F41" s="93"/>
+      <c r="G41" s="93"/>
+      <c r="H41" s="95" t="s">
         <v>144</v>
       </c>
-      <c r="I41" s="94"/>
-      <c r="J41" s="95"/>
-      <c r="K41" s="90" t="s">
+      <c r="I41" s="96"/>
+      <c r="J41" s="97"/>
+      <c r="K41" s="92" t="s">
         <v>145</v>
       </c>
-      <c r="L41" s="90"/>
-      <c r="M41" s="90"/>
-      <c r="N41" s="91">
+      <c r="L41" s="92"/>
+      <c r="M41" s="92"/>
+      <c r="N41" s="93">
         <v>400</v>
       </c>
-      <c r="O41" s="91"/>
-      <c r="P41" s="91"/>
-      <c r="Q41" s="90" t="s">
+      <c r="O41" s="93"/>
+      <c r="P41" s="93"/>
+      <c r="Q41" s="92" t="s">
         <v>146</v>
       </c>
-      <c r="R41" s="91"/>
-      <c r="S41" s="91"/>
-      <c r="T41" s="86" t="s">
+      <c r="R41" s="93"/>
+      <c r="S41" s="93"/>
+      <c r="T41" s="88" t="s">
         <v>48</v>
       </c>
-      <c r="U41" s="87"/>
-      <c r="V41" s="87"/>
-      <c r="W41" s="87"/>
+      <c r="U41" s="89"/>
+      <c r="V41" s="89"/>
+      <c r="W41" s="89"/>
     </row>
     <row r="42" ht="134.25" customHeight="1" spans="1:25">
-      <c r="A42" s="83" t="s">
+      <c r="A42" s="85" t="s">
         <v>61</v>
       </c>
-      <c r="B42" s="24"/>
-      <c r="C42" s="96" t="s">
+      <c r="B42" s="26"/>
+      <c r="C42" s="98" t="s">
         <v>147</v>
       </c>
-      <c r="D42" s="97"/>
-      <c r="E42" s="97"/>
-      <c r="F42" s="97"/>
-      <c r="G42" s="98"/>
-      <c r="H42" s="29" t="s">
+      <c r="D42" s="99"/>
+      <c r="E42" s="99"/>
+      <c r="F42" s="99"/>
+      <c r="G42" s="100"/>
+      <c r="H42" s="31" t="s">
         <v>148</v>
       </c>
-      <c r="I42" s="29"/>
-      <c r="J42" s="29"/>
-      <c r="K42" s="29" t="s">
+      <c r="I42" s="31"/>
+      <c r="J42" s="31"/>
+      <c r="K42" s="31" t="s">
         <v>149</v>
       </c>
-      <c r="L42" s="29"/>
-      <c r="M42" s="29"/>
-      <c r="N42" s="26">
+      <c r="L42" s="31"/>
+      <c r="M42" s="31"/>
+      <c r="N42" s="28">
         <v>200</v>
       </c>
-      <c r="O42" s="26"/>
-      <c r="P42" s="26"/>
-      <c r="Q42" s="26" t="s">
+      <c r="O42" s="28"/>
+      <c r="P42" s="28"/>
+      <c r="Q42" s="28" t="s">
         <v>150</v>
       </c>
-      <c r="R42" s="26"/>
-      <c r="S42" s="26"/>
-      <c r="T42" s="46" t="s">
+      <c r="R42" s="28"/>
+      <c r="S42" s="28"/>
+      <c r="T42" s="48" t="s">
         <v>125</v>
       </c>
-      <c r="U42" s="46"/>
-      <c r="V42" s="46"/>
-      <c r="W42" s="46"/>
+      <c r="U42" s="48"/>
+      <c r="V42" s="48"/>
+      <c r="W42" s="48"/>
     </row>
     <row r="43" ht="134.25" customHeight="1" spans="1:25">
-      <c r="A43" s="89"/>
-      <c r="B43" s="65"/>
-      <c r="C43" s="99" t="s">
+      <c r="A43" s="91"/>
+      <c r="B43" s="67"/>
+      <c r="C43" s="101" t="s">
         <v>147</v>
       </c>
-      <c r="D43" s="100"/>
-      <c r="E43" s="100"/>
-      <c r="F43" s="100"/>
-      <c r="G43" s="53"/>
-      <c r="H43" s="55" t="s">
+      <c r="D43" s="102"/>
+      <c r="E43" s="102"/>
+      <c r="F43" s="102"/>
+      <c r="G43" s="55"/>
+      <c r="H43" s="57" t="s">
         <v>151</v>
       </c>
-      <c r="I43" s="55"/>
-      <c r="J43" s="55"/>
-      <c r="K43" s="101" t="s">
+      <c r="I43" s="57"/>
+      <c r="J43" s="57"/>
+      <c r="K43" s="103" t="s">
         <v>152</v>
       </c>
-      <c r="L43" s="102"/>
-      <c r="M43" s="103"/>
-      <c r="N43" s="101" t="s">
+      <c r="L43" s="104"/>
+      <c r="M43" s="105"/>
+      <c r="N43" s="103" t="s">
         <v>153</v>
       </c>
-      <c r="O43" s="102"/>
-      <c r="P43" s="103"/>
-      <c r="Q43" s="99"/>
-      <c r="R43" s="100"/>
-      <c r="S43" s="53"/>
-      <c r="T43" s="101"/>
-      <c r="U43" s="102"/>
-      <c r="V43" s="102"/>
-      <c r="W43" s="103"/>
+      <c r="O43" s="104"/>
+      <c r="P43" s="105"/>
+      <c r="Q43" s="101"/>
+      <c r="R43" s="102"/>
+      <c r="S43" s="55"/>
+      <c r="T43" s="103"/>
+      <c r="U43" s="104"/>
+      <c r="V43" s="104"/>
+      <c r="W43" s="105"/>
     </row>
     <row r="44" ht="134.25" customHeight="1" spans="1:25">
-      <c r="A44" s="83" t="s">
+      <c r="A44" s="85" t="s">
         <v>74</v>
       </c>
-      <c r="B44" s="83"/>
-      <c r="C44" s="92" t="s">
+      <c r="B44" s="85"/>
+      <c r="C44" s="94" t="s">
         <v>140</v>
       </c>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
-      <c r="F44" s="92"/>
-      <c r="G44" s="92"/>
-      <c r="H44" s="59" t="s">
+      <c r="D44" s="94"/>
+      <c r="E44" s="94"/>
+      <c r="F44" s="94"/>
+      <c r="G44" s="94"/>
+      <c r="H44" s="61" t="s">
         <v>154</v>
       </c>
-      <c r="I44" s="60"/>
-      <c r="J44" s="61"/>
-      <c r="K44" s="30" t="s">
+      <c r="I44" s="62"/>
+      <c r="J44" s="63"/>
+      <c r="K44" s="32" t="s">
         <v>155</v>
       </c>
-      <c r="L44" s="62"/>
-      <c r="M44" s="63"/>
-      <c r="N44" s="26">
+      <c r="L44" s="64"/>
+      <c r="M44" s="65"/>
+      <c r="N44" s="28">
         <v>200</v>
       </c>
-      <c r="O44" s="26"/>
-      <c r="P44" s="26"/>
-      <c r="Q44" s="26" t="s">
+      <c r="O44" s="28"/>
+      <c r="P44" s="28"/>
+      <c r="Q44" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="R44" s="26"/>
-      <c r="S44" s="26"/>
-      <c r="T44" s="46" t="s">
+      <c r="R44" s="28"/>
+      <c r="S44" s="28"/>
+      <c r="T44" s="48" t="s">
         <v>78</v>
       </c>
-      <c r="U44" s="46"/>
-      <c r="V44" s="46"/>
-      <c r="W44" s="46"/>
+      <c r="U44" s="48"/>
+      <c r="V44" s="48"/>
+      <c r="W44" s="48"/>
     </row>
     <row r="45" ht="117" customHeight="1" spans="1:25">
-      <c r="A45" s="23" t="s">
+      <c r="A45" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="B45" s="24"/>
-      <c r="C45" s="92" t="s">
+      <c r="B45" s="26"/>
+      <c r="C45" s="94" t="s">
         <v>147</v>
       </c>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
-      <c r="F45" s="92"/>
-      <c r="G45" s="92"/>
-      <c r="H45" s="59" t="s">
+      <c r="D45" s="94"/>
+      <c r="E45" s="94"/>
+      <c r="F45" s="94"/>
+      <c r="G45" s="94"/>
+      <c r="H45" s="61" t="s">
         <v>156</v>
       </c>
-      <c r="I45" s="60"/>
-      <c r="J45" s="61"/>
-      <c r="K45" s="29" t="s">
+      <c r="I45" s="62"/>
+      <c r="J45" s="63"/>
+      <c r="K45" s="31" t="s">
         <v>157</v>
       </c>
-      <c r="L45" s="29"/>
-      <c r="M45" s="29"/>
-      <c r="N45" s="26">
+      <c r="L45" s="31"/>
+      <c r="M45" s="31"/>
+      <c r="N45" s="28">
         <v>200</v>
       </c>
-      <c r="O45" s="26"/>
-      <c r="P45" s="26"/>
-      <c r="Q45" s="26" t="s">
+      <c r="O45" s="28"/>
+      <c r="P45" s="28"/>
+      <c r="Q45" s="28" t="s">
         <v>158</v>
       </c>
-      <c r="R45" s="26"/>
-      <c r="S45" s="26"/>
-      <c r="T45" s="46" t="s">
+      <c r="R45" s="28"/>
+      <c r="S45" s="28"/>
+      <c r="T45" s="48" t="s">
         <v>116</v>
       </c>
-      <c r="U45" s="46"/>
-      <c r="V45" s="46"/>
-      <c r="W45" s="46"/>
+      <c r="U45" s="48"/>
+      <c r="V45" s="48"/>
+      <c r="W45" s="48"/>
     </row>
     <row r="46" ht="195" customHeight="1" spans="1:25">
-      <c r="A46" s="33"/>
-      <c r="B46" s="34"/>
-      <c r="C46" s="92" t="s">
+      <c r="A46" s="35"/>
+      <c r="B46" s="36"/>
+      <c r="C46" s="94" t="s">
         <v>147</v>
       </c>
-      <c r="D46" s="92"/>
-      <c r="E46" s="92"/>
-      <c r="F46" s="92"/>
-      <c r="G46" s="92"/>
-      <c r="H46" s="67" t="s">
+      <c r="D46" s="94"/>
+      <c r="E46" s="94"/>
+      <c r="F46" s="94"/>
+      <c r="G46" s="94"/>
+      <c r="H46" s="69" t="s">
         <v>159</v>
       </c>
-      <c r="I46" s="68"/>
-      <c r="J46" s="69"/>
-      <c r="K46" s="36" t="s">
+      <c r="I46" s="70"/>
+      <c r="J46" s="71"/>
+      <c r="K46" s="38" t="s">
         <v>160</v>
       </c>
-      <c r="L46" s="36"/>
-      <c r="M46" s="36"/>
+      <c r="L46" s="38"/>
+      <c r="M46" s="38"/>
       <c r="N46" s="4">
         <v>400</v>
       </c>
       <c r="O46" s="4"/>
       <c r="P46" s="4"/>
-      <c r="Q46" s="70" t="s">
+      <c r="Q46" s="72" t="s">
         <v>161</v>
       </c>
-      <c r="R46" s="71"/>
-      <c r="S46" s="72"/>
-      <c r="T46" s="37" t="s">
+      <c r="R46" s="73"/>
+      <c r="S46" s="74"/>
+      <c r="T46" s="39" t="s">
         <v>86</v>
       </c>
-      <c r="U46" s="37"/>
-      <c r="V46" s="37"/>
-      <c r="W46" s="37"/>
-      <c r="Y46" s="104"/>
+      <c r="U46" s="39"/>
+      <c r="V46" s="39"/>
+      <c r="W46" s="39"/>
+      <c r="Y46" s="106"/>
     </row>
     <row r="47" ht="195" customHeight="1" spans="1:25">
-      <c r="A47" s="33"/>
-      <c r="B47" s="34"/>
-      <c r="C47" s="92" t="s">
+      <c r="A47" s="35"/>
+      <c r="B47" s="36"/>
+      <c r="C47" s="94" t="s">
         <v>162</v>
       </c>
-      <c r="D47" s="92"/>
-      <c r="E47" s="92"/>
-      <c r="F47" s="92"/>
-      <c r="G47" s="92"/>
-      <c r="H47" s="67" t="s">
+      <c r="D47" s="94"/>
+      <c r="E47" s="94"/>
+      <c r="F47" s="94"/>
+      <c r="G47" s="94"/>
+      <c r="H47" s="69" t="s">
         <v>163</v>
       </c>
-      <c r="I47" s="68"/>
-      <c r="J47" s="69"/>
-      <c r="K47" s="36" t="s">
+      <c r="I47" s="70"/>
+      <c r="J47" s="71"/>
+      <c r="K47" s="38" t="s">
         <v>164</v>
       </c>
-      <c r="L47" s="36"/>
-      <c r="M47" s="36"/>
+      <c r="L47" s="38"/>
+      <c r="M47" s="38"/>
       <c r="N47" s="4">
         <v>200</v>
       </c>
       <c r="O47" s="4"/>
       <c r="P47" s="4"/>
-      <c r="Q47" s="26" t="s">
+      <c r="Q47" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="R47" s="26"/>
-      <c r="S47" s="26"/>
-      <c r="T47" s="46" t="s">
+      <c r="R47" s="28"/>
+      <c r="S47" s="28"/>
+      <c r="T47" s="48" t="s">
         <v>78</v>
       </c>
-      <c r="U47" s="46"/>
-      <c r="V47" s="46"/>
-      <c r="W47" s="46"/>
-      <c r="Y47" s="104"/>
+      <c r="U47" s="48"/>
+      <c r="V47" s="48"/>
+      <c r="W47" s="48"/>
+      <c r="Y47" s="106"/>
     </row>
     <row r="48" ht="221.25" customHeight="1" spans="1:25">
-      <c r="A48" s="64"/>
-      <c r="B48" s="65"/>
-      <c r="C48" s="92" t="s">
+      <c r="A48" s="66"/>
+      <c r="B48" s="67"/>
+      <c r="C48" s="94" t="s">
         <v>162</v>
       </c>
-      <c r="D48" s="92"/>
-      <c r="E48" s="92"/>
-      <c r="F48" s="92"/>
-      <c r="G48" s="92"/>
-      <c r="H48" s="67" t="s">
+      <c r="D48" s="94"/>
+      <c r="E48" s="94"/>
+      <c r="F48" s="94"/>
+      <c r="G48" s="94"/>
+      <c r="H48" s="69" t="s">
         <v>163</v>
       </c>
-      <c r="I48" s="68"/>
-      <c r="J48" s="69"/>
-      <c r="K48" s="36" t="s">
+      <c r="I48" s="70"/>
+      <c r="J48" s="71"/>
+      <c r="K48" s="38" t="s">
         <v>165</v>
       </c>
-      <c r="L48" s="36"/>
-      <c r="M48" s="36"/>
+      <c r="L48" s="38"/>
+      <c r="M48" s="38"/>
       <c r="N48" s="4">
         <v>400</v>
       </c>
       <c r="O48" s="4"/>
       <c r="P48" s="4"/>
-      <c r="Q48" s="70" t="s">
+      <c r="Q48" s="72" t="s">
         <v>166</v>
       </c>
-      <c r="R48" s="71"/>
-      <c r="S48" s="72"/>
-      <c r="T48" s="37" t="s">
+      <c r="R48" s="73"/>
+      <c r="S48" s="74"/>
+      <c r="T48" s="39" t="s">
         <v>86</v>
       </c>
-      <c r="U48" s="37"/>
-      <c r="V48" s="37"/>
-      <c r="W48" s="37"/>
+      <c r="U48" s="39"/>
+      <c r="V48" s="39"/>
+      <c r="W48" s="39"/>
     </row>
     <row r="49" ht="60" customHeight="1" spans="1:23">
       <c r="A49" s="4" t="s">
         <v>87</v>
       </c>
       <c r="B49" s="4"/>
-      <c r="C49" s="92" t="s">
+      <c r="C49" s="94" t="s">
         <v>147</v>
       </c>
-      <c r="D49" s="92"/>
-      <c r="E49" s="92"/>
-      <c r="F49" s="92"/>
-      <c r="G49" s="92"/>
-      <c r="H49" s="29" t="s">
+      <c r="D49" s="94"/>
+      <c r="E49" s="94"/>
+      <c r="F49" s="94"/>
+      <c r="G49" s="94"/>
+      <c r="H49" s="31" t="s">
         <v>167</v>
       </c>
-      <c r="I49" s="29"/>
-      <c r="J49" s="29"/>
-      <c r="K49" s="29" t="s">
+      <c r="I49" s="31"/>
+      <c r="J49" s="31"/>
+      <c r="K49" s="31" t="s">
         <v>168</v>
       </c>
-      <c r="L49" s="29"/>
-      <c r="M49" s="29"/>
-      <c r="N49" s="26">
+      <c r="L49" s="31"/>
+      <c r="M49" s="31"/>
+      <c r="N49" s="28">
         <v>200</v>
       </c>
-      <c r="O49" s="26"/>
-      <c r="P49" s="26"/>
-      <c r="Q49" s="26" t="s">
+      <c r="O49" s="28"/>
+      <c r="P49" s="28"/>
+      <c r="Q49" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="R49" s="26"/>
-      <c r="S49" s="26"/>
-      <c r="T49" s="46" t="s">
+      <c r="R49" s="28"/>
+      <c r="S49" s="28"/>
+      <c r="T49" s="48" t="s">
         <v>91</v>
       </c>
-      <c r="U49" s="73"/>
-      <c r="V49" s="73"/>
-      <c r="W49" s="73"/>
+      <c r="U49" s="75"/>
+      <c r="V49" s="75"/>
+      <c r="W49" s="75"/>
     </row>
     <row r="50" ht="218.25" customHeight="1" spans="1:23">
       <c r="A50" s="4"/>
       <c r="B50" s="4"/>
-      <c r="C50" s="92" t="s">
+      <c r="C50" s="94" t="s">
         <v>147</v>
       </c>
-      <c r="D50" s="92"/>
-      <c r="E50" s="92"/>
-      <c r="F50" s="92"/>
-      <c r="G50" s="92"/>
-      <c r="H50" s="37" t="s">
+      <c r="D50" s="94"/>
+      <c r="E50" s="94"/>
+      <c r="F50" s="94"/>
+      <c r="G50" s="94"/>
+      <c r="H50" s="39" t="s">
         <v>169</v>
       </c>
-      <c r="I50" s="37"/>
-      <c r="J50" s="37"/>
-      <c r="K50" s="36" t="s">
+      <c r="I50" s="39"/>
+      <c r="J50" s="39"/>
+      <c r="K50" s="38" t="s">
         <v>170</v>
       </c>
-      <c r="L50" s="36"/>
-      <c r="M50" s="36"/>
+      <c r="L50" s="38"/>
+      <c r="M50" s="38"/>
       <c r="N50" s="4">
         <v>400</v>
       </c>
       <c r="O50" s="4"/>
       <c r="P50" s="4"/>
-      <c r="Q50" s="39" t="s">
+      <c r="Q50" s="41" t="s">
         <v>171</v>
       </c>
-      <c r="R50" s="39"/>
-      <c r="S50" s="39"/>
-      <c r="T50" s="37" t="s">
+      <c r="R50" s="41"/>
+      <c r="S50" s="41"/>
+      <c r="T50" s="39" t="s">
         <v>86</v>
       </c>
-      <c r="U50" s="37"/>
-      <c r="V50" s="37"/>
-      <c r="W50" s="37"/>
+      <c r="U50" s="39"/>
+      <c r="V50" s="39"/>
+      <c r="W50" s="39"/>
     </row>
     <row r="51" spans="1:23">
-      <c r="A51" s="15" t="s">
+      <c r="A51" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="B51" s="16"/>
-      <c r="C51" s="16"/>
-      <c r="D51" s="16"/>
-      <c r="E51" s="16"/>
-      <c r="F51" s="16"/>
-      <c r="G51" s="16"/>
-      <c r="H51" s="16"/>
-      <c r="I51" s="16"/>
-      <c r="J51" s="16"/>
-      <c r="K51" s="16"/>
-      <c r="L51" s="16"/>
-      <c r="M51" s="16"/>
-      <c r="N51" s="16"/>
-      <c r="O51" s="16"/>
-      <c r="P51" s="16"/>
-      <c r="Q51" s="16"/>
-      <c r="R51" s="16"/>
-      <c r="S51" s="16"/>
-      <c r="T51" s="16"/>
-      <c r="U51" s="16"/>
-      <c r="V51" s="16"/>
-      <c r="W51" s="17"/>
-    </row>
-    <row r="52" spans="1:23">
-      <c r="A52" s="105"/>
-      <c r="B52" s="105"/>
-    </row>
-    <row r="53" spans="1:23">
-      <c r="A53" s="105"/>
-      <c r="B53" s="105"/>
-      <c r="R53" s="106"/>
-    </row>
-    <row r="54" spans="1:23">
-      <c r="A54" s="105"/>
-      <c r="B54" s="105"/>
-    </row>
-    <row r="55" spans="1:23">
-      <c r="A55" s="105"/>
-      <c r="B55" s="105"/>
+      <c r="B51" s="18"/>
+      <c r="C51" s="18"/>
+      <c r="D51" s="18"/>
+      <c r="E51" s="18"/>
+      <c r="F51" s="18"/>
+      <c r="G51" s="18"/>
+      <c r="H51" s="18"/>
+      <c r="I51" s="18"/>
+      <c r="J51" s="18"/>
+      <c r="K51" s="18"/>
+      <c r="L51" s="18"/>
+      <c r="M51" s="18"/>
+      <c r="N51" s="18"/>
+      <c r="O51" s="18"/>
+      <c r="P51" s="18"/>
+      <c r="Q51" s="18"/>
+      <c r="R51" s="18"/>
+      <c r="S51" s="18"/>
+      <c r="T51" s="18"/>
+      <c r="U51" s="18"/>
+      <c r="V51" s="18"/>
+      <c r="W51" s="19"/>
+    </row>
+    <row r="52" ht="113" customHeight="1" spans="1:23">
+      <c r="A52" s="107" t="s">
+        <v>74</v>
+      </c>
+      <c r="B52" s="107"/>
+      <c r="C52" s="108" t="s">
+        <v>173</v>
+      </c>
+      <c r="D52" s="108"/>
+      <c r="E52" s="108"/>
+      <c r="F52" s="108"/>
+      <c r="G52" s="108"/>
+      <c r="H52" s="109" t="s">
+        <v>174</v>
+      </c>
+      <c r="I52" s="110"/>
+      <c r="J52" s="111"/>
+      <c r="K52" s="112" t="s">
+        <v>175</v>
+      </c>
+      <c r="L52" s="113"/>
+      <c r="M52" s="114"/>
+      <c r="N52" s="108">
+        <v>200</v>
+      </c>
+      <c r="O52" s="108"/>
+      <c r="P52" s="108"/>
+      <c r="Q52" s="108" t="s">
+        <v>176</v>
+      </c>
+      <c r="R52" s="108"/>
+      <c r="S52" s="108"/>
+      <c r="T52" s="115" t="s">
+        <v>177</v>
+      </c>
+      <c r="U52" s="115"/>
+      <c r="V52" s="115"/>
+      <c r="W52" s="115"/>
+    </row>
+    <row r="53" ht="125" customHeight="1" spans="1:23">
+      <c r="A53" s="107"/>
+      <c r="B53" s="107"/>
+      <c r="C53" s="108" t="s">
+        <v>178</v>
+      </c>
+      <c r="D53" s="108"/>
+      <c r="E53" s="108"/>
+      <c r="F53" s="108"/>
+      <c r="G53" s="108"/>
+      <c r="H53" s="109" t="s">
+        <v>179</v>
+      </c>
+      <c r="I53" s="110"/>
+      <c r="J53" s="111"/>
+      <c r="K53" s="112" t="s">
+        <v>180</v>
+      </c>
+      <c r="L53" s="113"/>
+      <c r="M53" s="114"/>
+      <c r="N53" s="108">
+        <v>200</v>
+      </c>
+      <c r="O53" s="108"/>
+      <c r="P53" s="108"/>
+      <c r="Q53" s="108" t="s">
+        <v>176</v>
+      </c>
+      <c r="R53" s="108"/>
+      <c r="S53" s="108"/>
+      <c r="T53" s="115" t="s">
+        <v>181</v>
+      </c>
+      <c r="U53" s="115"/>
+      <c r="V53" s="115"/>
+      <c r="W53" s="115"/>
+    </row>
+    <row r="54" ht="101" customHeight="1" spans="1:23">
+      <c r="A54" s="107"/>
+      <c r="B54" s="107"/>
+      <c r="C54" s="108" t="s">
+        <v>182</v>
+      </c>
+      <c r="D54" s="108"/>
+      <c r="E54" s="108"/>
+      <c r="F54" s="108"/>
+      <c r="G54" s="108"/>
+      <c r="H54" s="109" t="s">
+        <v>183</v>
+      </c>
+      <c r="I54" s="110"/>
+      <c r="J54" s="111"/>
+      <c r="K54" s="112" t="s">
+        <v>180</v>
+      </c>
+      <c r="L54" s="113"/>
+      <c r="M54" s="114"/>
+      <c r="N54" s="108">
+        <v>200</v>
+      </c>
+      <c r="O54" s="108"/>
+      <c r="P54" s="108"/>
+      <c r="Q54" s="108" t="s">
+        <v>176</v>
+      </c>
+      <c r="R54" s="108"/>
+      <c r="S54" s="108"/>
+      <c r="T54" s="115" t="s">
+        <v>181</v>
+      </c>
+      <c r="U54" s="115"/>
+      <c r="V54" s="115"/>
+      <c r="W54" s="115"/>
+    </row>
+    <row r="55" ht="65" customHeight="1" spans="1:23">
+      <c r="A55" s="107"/>
+      <c r="B55" s="107"/>
+      <c r="C55" s="108" t="s">
+        <v>184</v>
+      </c>
+      <c r="D55" s="108"/>
+      <c r="E55" s="108"/>
+      <c r="F55" s="108"/>
+      <c r="G55" s="108"/>
+      <c r="H55" s="109" t="s">
+        <v>183</v>
+      </c>
+      <c r="I55" s="110"/>
+      <c r="J55" s="111"/>
+      <c r="K55" s="112" t="s">
+        <v>185</v>
+      </c>
+      <c r="L55" s="113"/>
+      <c r="M55" s="114"/>
+      <c r="N55" s="108">
+        <v>200</v>
+      </c>
+      <c r="O55" s="108"/>
+      <c r="P55" s="108"/>
+      <c r="Q55" s="108" t="s">
+        <v>176</v>
+      </c>
+      <c r="R55" s="108"/>
+      <c r="S55" s="108"/>
+      <c r="T55" s="115" t="s">
+        <v>181</v>
+      </c>
+      <c r="U55" s="115"/>
+      <c r="V55" s="115"/>
+      <c r="W55" s="115"/>
+    </row>
+    <row r="56" ht="82" customHeight="1" spans="1:23">
+      <c r="A56" s="107"/>
+      <c r="B56" s="107"/>
+      <c r="C56" s="108" t="s">
+        <v>186</v>
+      </c>
+      <c r="D56" s="108"/>
+      <c r="E56" s="108"/>
+      <c r="F56" s="108"/>
+      <c r="G56" s="108"/>
+      <c r="H56" s="109" t="s">
+        <v>187</v>
+      </c>
+      <c r="I56" s="110"/>
+      <c r="J56" s="111"/>
+      <c r="K56" s="112" t="s">
+        <v>188</v>
+      </c>
+      <c r="L56" s="113"/>
+      <c r="M56" s="114"/>
+      <c r="N56" s="108">
+        <v>200</v>
+      </c>
+      <c r="O56" s="108"/>
+      <c r="P56" s="108"/>
+      <c r="Q56" s="108" t="s">
+        <v>176</v>
+      </c>
+      <c r="R56" s="108"/>
+      <c r="S56" s="108"/>
+      <c r="T56" s="115" t="s">
+        <v>189</v>
+      </c>
+      <c r="U56" s="115"/>
+      <c r="V56" s="115"/>
+      <c r="W56" s="115"/>
+    </row>
+    <row r="59" spans="1:23">
+      <c r="U59" s="15" t="s">
+        <v>190</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="261">
+  <mergeCells count="292">
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="A2:W2"/>
     <mergeCell ref="A3:B3"/>
@@ -4471,6 +4749,36 @@
     <mergeCell ref="Q50:S50"/>
     <mergeCell ref="T50:W50"/>
     <mergeCell ref="A51:W51"/>
+    <mergeCell ref="C52:G52"/>
+    <mergeCell ref="H52:J52"/>
+    <mergeCell ref="K52:M52"/>
+    <mergeCell ref="N52:P52"/>
+    <mergeCell ref="Q52:S52"/>
+    <mergeCell ref="T52:W52"/>
+    <mergeCell ref="C53:G53"/>
+    <mergeCell ref="H53:J53"/>
+    <mergeCell ref="K53:M53"/>
+    <mergeCell ref="N53:P53"/>
+    <mergeCell ref="Q53:S53"/>
+    <mergeCell ref="T53:W53"/>
+    <mergeCell ref="C54:G54"/>
+    <mergeCell ref="H54:J54"/>
+    <mergeCell ref="K54:M54"/>
+    <mergeCell ref="N54:P54"/>
+    <mergeCell ref="Q54:S54"/>
+    <mergeCell ref="T54:W54"/>
+    <mergeCell ref="C55:G55"/>
+    <mergeCell ref="H55:J55"/>
+    <mergeCell ref="K55:M55"/>
+    <mergeCell ref="N55:P55"/>
+    <mergeCell ref="Q55:S55"/>
+    <mergeCell ref="T55:W55"/>
+    <mergeCell ref="C56:G56"/>
+    <mergeCell ref="H56:J56"/>
+    <mergeCell ref="K56:M56"/>
+    <mergeCell ref="N56:P56"/>
+    <mergeCell ref="Q56:S56"/>
+    <mergeCell ref="T56:W56"/>
     <mergeCell ref="A49:B50"/>
     <mergeCell ref="A45:B48"/>
     <mergeCell ref="A42:B43"/>
@@ -4489,6 +4797,7 @@
     <mergeCell ref="A10:B19"/>
     <mergeCell ref="T10:W16"/>
     <mergeCell ref="A21:B22"/>
+    <mergeCell ref="A52:B56"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C20" r:id="rId1" display="/api/v1/products/"/>
@@ -4512,7 +4821,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="B1" s="1" t="s">
-        <v>173</v>
+        <v>191</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -4527,53 +4836,53 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="2" t="s">
-        <v>174</v>
+        <v>192</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>177</v>
+        <v>195</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>178</v>
+        <v>196</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>179</v>
+        <v>197</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>180</v>
+        <v>198</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>181</v>
+        <v>199</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>182</v>
+        <v>200</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>183</v>
+        <v>201</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>185</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" s="6" t="s">
-        <v>186</v>
+        <v>204</v>
       </c>
       <c r="B3" s="3">
         <v>1</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="7">
         <v>1</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="7">
         <v>0</v>
       </c>
       <c r="E3" s="3">
@@ -4594,7 +4903,7 @@
       <c r="J3" s="3">
         <v>1</v>
       </c>
-      <c r="K3" s="7">
+      <c r="K3" s="8">
         <v>1</v>
       </c>
       <c r="L3" s="3">
@@ -4603,15 +4912,15 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="6" t="s">
-        <v>187</v>
+        <v>205</v>
       </c>
       <c r="B4" s="3">
         <v>1</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="7">
         <v>0</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="7">
         <v>1</v>
       </c>
       <c r="E4" s="3">
@@ -4626,7 +4935,7 @@
       <c r="H4" s="3">
         <v>1</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="9">
         <v>1</v>
       </c>
       <c r="J4" s="3">
@@ -4641,15 +4950,15 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="6" t="s">
-        <v>188</v>
+        <v>206</v>
       </c>
       <c r="B5" s="3">
         <v>1</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="7">
         <v>0</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="7">
         <v>0</v>
       </c>
       <c r="E5" s="3">
@@ -4664,7 +4973,7 @@
       <c r="H5" s="3">
         <v>0</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="9">
         <v>1</v>
       </c>
       <c r="J5" s="3">
@@ -4679,15 +4988,15 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" s="6" t="s">
-        <v>189</v>
+        <v>207</v>
       </c>
       <c r="B6" s="3">
         <v>1</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="7">
         <v>0</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="7">
         <v>0</v>
       </c>
       <c r="E6" s="3">
@@ -4711,21 +5020,21 @@
       <c r="K6" s="3">
         <v>0</v>
       </c>
-      <c r="L6" s="8">
+      <c r="L6" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="6" t="s">
-        <v>190</v>
+        <v>208</v>
       </c>
       <c r="B7" s="3">
         <v>1</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="7">
         <v>0</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="7">
         <v>0</v>
       </c>
       <c r="E7" s="3">
@@ -4746,56 +5055,56 @@
       <c r="J7" s="3">
         <v>0</v>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="8">
         <v>1</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:12">
-      <c r="A8" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
+      <c r="A8" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="B8" s="10"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="6" t="s">
-        <v>192</v>
+        <v>210</v>
       </c>
       <c r="B9" s="3">
         <v>1</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="7">
         <v>1</v>
       </c>
-      <c r="D9" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="E9" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="F9" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="G9" s="113" t="s">
-        <v>193</v>
+      <c r="D9" s="122" t="s">
+        <v>211</v>
+      </c>
+      <c r="E9" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="F9" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="G9" s="123" t="s">
+        <v>211</v>
       </c>
       <c r="H9" s="3">
         <v>1</v>
       </c>
-      <c r="I9" s="113" t="s">
-        <v>193</v>
+      <c r="I9" s="123" t="s">
+        <v>211</v>
       </c>
       <c r="J9" s="3">
         <v>1</v>
@@ -4803,31 +5112,31 @@
       <c r="K9" s="3">
         <v>1</v>
       </c>
-      <c r="L9" s="113" t="s">
-        <v>193</v>
+      <c r="L9" s="123" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="6" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="D10" s="3">
+      <c r="C10" s="122" t="s">
+        <v>211</v>
+      </c>
+      <c r="D10" s="7">
         <v>1</v>
       </c>
-      <c r="E10" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="F10" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="G10" s="113" t="s">
-        <v>193</v>
+      <c r="E10" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="F10" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="G10" s="123" t="s">
+        <v>211</v>
       </c>
       <c r="H10" s="3">
         <v>1</v>
@@ -4835,125 +5144,125 @@
       <c r="I10" s="3">
         <v>1</v>
       </c>
-      <c r="J10" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="K10" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="L10" s="113" t="s">
-        <v>193</v>
+      <c r="J10" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="K10" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="L10" s="123" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="6" t="s">
-        <v>195</v>
+        <v>213</v>
       </c>
       <c r="B11" s="3">
         <v>1</v>
       </c>
-      <c r="C11" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="D11" s="113" t="s">
-        <v>193</v>
+      <c r="C11" s="122" t="s">
+        <v>211</v>
+      </c>
+      <c r="D11" s="122" t="s">
+        <v>211</v>
       </c>
       <c r="E11" s="3">
         <v>1</v>
       </c>
-      <c r="F11" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="G11" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="H11" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="I11" s="113" t="s">
-        <v>193</v>
+      <c r="F11" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="G11" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="H11" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="I11" s="123" t="s">
+        <v>211</v>
       </c>
       <c r="J11" s="3">
         <v>1</v>
       </c>
-      <c r="K11" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="L11" s="113" t="s">
-        <v>193</v>
+      <c r="K11" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="L11" s="123" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="6" t="s">
-        <v>196</v>
+        <v>214</v>
       </c>
       <c r="B12" s="3">
         <v>1</v>
       </c>
-      <c r="C12" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="D12" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="E12" s="113" t="s">
-        <v>193</v>
+      <c r="C12" s="122" t="s">
+        <v>211</v>
+      </c>
+      <c r="D12" s="122" t="s">
+        <v>211</v>
+      </c>
+      <c r="E12" s="123" t="s">
+        <v>211</v>
       </c>
       <c r="F12" s="3">
         <v>1</v>
       </c>
-      <c r="G12" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="H12" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="I12" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="J12" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="K12" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="L12" s="113" t="s">
-        <v>193</v>
+      <c r="G12" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="H12" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="I12" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="J12" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="K12" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="L12" s="123" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="6" t="s">
-        <v>197</v>
+        <v>215</v>
       </c>
       <c r="B13" s="3">
         <v>1</v>
       </c>
-      <c r="C13" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="D13" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="E13" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="F13" s="113" t="s">
-        <v>193</v>
+      <c r="C13" s="122" t="s">
+        <v>211</v>
+      </c>
+      <c r="D13" s="122" t="s">
+        <v>211</v>
+      </c>
+      <c r="E13" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="F13" s="123" t="s">
+        <v>211</v>
       </c>
       <c r="G13" s="3">
         <v>1</v>
       </c>
-      <c r="H13" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="I13" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="J13" s="113" t="s">
-        <v>193</v>
-      </c>
-      <c r="K13" s="113" t="s">
-        <v>193</v>
+      <c r="H13" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="I13" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="J13" s="123" t="s">
+        <v>211</v>
+      </c>
+      <c r="K13" s="123" t="s">
+        <v>211</v>
       </c>
       <c r="L13" s="3">
         <v>1</v>
@@ -4968,15 +5277,15 @@
       <c r="F14" s="6"/>
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
-      <c r="I14" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="J14" s="11"/>
-      <c r="K14" s="10" t="s">
-        <v>199</v>
-      </c>
-      <c r="L14" s="10" t="s">
-        <v>200</v>
+      <c r="I14" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="J14" s="13"/>
+      <c r="K14" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="L14" s="12" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs:actualizando archivo segumiento automatización
</commit_message>
<xml_diff>
--- a/Plan_de_pruebas_analisis.xlsx
+++ b/Plan_de_pruebas_analisis.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11580" activeTab="3"/>
+    <workbookView windowWidth="28800" windowHeight="12180" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Back" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="225">
   <si>
     <t>BackEnd</t>
   </si>
@@ -752,6 +752,15 @@
 * Validar que en la respuesta los productos esten realacionado con el precio  buscado</t>
   </si>
   <si>
+    <t>Consulta la lista de todos los productos por precio no existente</t>
+  </si>
+  <si>
+    <t>* Validar que el servicio no retorne resultado si se consulta por precio no existente</t>
+  </si>
+  <si>
+    <t>Lista vacia de productos</t>
+  </si>
+  <si>
     <t>/api/v1/products/?price_min&amp;price_max</t>
   </si>
   <si>
@@ -777,6 +786,18 @@
 * Validar contrato de la respuesta para cada elemento. 
 * Validar codigo de estado.
 * Validar que en la respuesta los productos esten realacionado con el id  buscado</t>
+  </si>
+  <si>
+    <t>Consulta la lista por categoria por un Id que no existe</t>
+  </si>
+  <si>
+    <t>* Validar que el servicio no retorne resultado si se consulta por una categoria que no existe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+* Validar que no retorne prodcutos 
+* Validar codigo de estado.
+</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -1165,6 +1186,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1268,12 +1295,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1544,7 +1565,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1568,14 +1589,14 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="19" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="20" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="13" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1587,22 +1608,22 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1611,22 +1632,22 @@
     <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1635,21 +1656,21 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -1660,7 +1681,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1973,28 +1994,34 @@
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2354,7 +2381,7 @@
       </c>
     </row>
     <row r="3" ht="90" spans="1:2">
-      <c r="B3" s="120" t="s">
+      <c r="B3" s="122" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2404,7 +2431,7 @@
       </c>
     </row>
     <row r="17" spans="2:2">
-      <c r="B17" s="121" t="s">
+      <c r="B17" s="123" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2443,22 +2470,22 @@
       <c r="A2" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="116" t="s">
+      <c r="B2" s="118" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" ht="30" spans="1:2">
-      <c r="B3" s="117" t="s">
+      <c r="B3" s="119" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" ht="30" spans="1:2">
-      <c r="B4" s="117" t="s">
+      <c r="B4" s="119" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="B9" s="118" t="s">
+      <c r="B9" s="120" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2483,27 +2510,27 @@
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="B16" s="119" t="s">
+      <c r="B16" s="121" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="17" ht="45" spans="2:2">
-      <c r="B17" s="120" t="s">
+      <c r="B17" s="122" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="18" ht="30" spans="2:2">
-      <c r="B18" s="120" t="s">
+      <c r="B18" s="122" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="19" ht="30" spans="2:2">
-      <c r="B19" s="117" t="s">
+      <c r="B19" s="119" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="20" ht="30" spans="2:2">
-      <c r="B20" s="120" t="s">
+      <c r="B20" s="122" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2516,7 +2543,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Y59"/>
+  <dimension ref="A1:Y60"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="19" width="11.4285714285714" style="14"/>
@@ -4320,36 +4347,36 @@
       <c r="C52" s="108" t="s">
         <v>173</v>
       </c>
-      <c r="D52" s="108"/>
-      <c r="E52" s="108"/>
-      <c r="F52" s="108"/>
-      <c r="G52" s="108"/>
-      <c r="H52" s="109" t="s">
+      <c r="D52" s="109"/>
+      <c r="E52" s="109"/>
+      <c r="F52" s="109"/>
+      <c r="G52" s="109"/>
+      <c r="H52" s="110" t="s">
         <v>174</v>
       </c>
-      <c r="I52" s="110"/>
-      <c r="J52" s="111"/>
-      <c r="K52" s="112" t="s">
+      <c r="I52" s="111"/>
+      <c r="J52" s="112"/>
+      <c r="K52" s="113" t="s">
         <v>175</v>
       </c>
-      <c r="L52" s="113"/>
-      <c r="M52" s="114"/>
-      <c r="N52" s="108">
+      <c r="L52" s="114"/>
+      <c r="M52" s="115"/>
+      <c r="N52" s="116">
         <v>200</v>
       </c>
-      <c r="O52" s="108"/>
-      <c r="P52" s="108"/>
-      <c r="Q52" s="108" t="s">
+      <c r="O52" s="116"/>
+      <c r="P52" s="116"/>
+      <c r="Q52" s="109" t="s">
         <v>176</v>
       </c>
-      <c r="R52" s="108"/>
-      <c r="S52" s="108"/>
-      <c r="T52" s="115" t="s">
+      <c r="R52" s="109"/>
+      <c r="S52" s="109"/>
+      <c r="T52" s="117" t="s">
         <v>177</v>
       </c>
-      <c r="U52" s="115"/>
-      <c r="V52" s="115"/>
-      <c r="W52" s="115"/>
+      <c r="U52" s="117"/>
+      <c r="V52" s="117"/>
+      <c r="W52" s="117"/>
     </row>
     <row r="53" ht="125" customHeight="1" spans="1:23">
       <c r="A53" s="107"/>
@@ -4357,155 +4384,229 @@
       <c r="C53" s="108" t="s">
         <v>178</v>
       </c>
-      <c r="D53" s="108"/>
-      <c r="E53" s="108"/>
-      <c r="F53" s="108"/>
-      <c r="G53" s="108"/>
-      <c r="H53" s="109" t="s">
+      <c r="D53" s="109"/>
+      <c r="E53" s="109"/>
+      <c r="F53" s="109"/>
+      <c r="G53" s="109"/>
+      <c r="H53" s="110" t="s">
         <v>179</v>
       </c>
-      <c r="I53" s="110"/>
-      <c r="J53" s="111"/>
-      <c r="K53" s="112" t="s">
+      <c r="I53" s="111"/>
+      <c r="J53" s="112"/>
+      <c r="K53" s="113" t="s">
         <v>180</v>
       </c>
-      <c r="L53" s="113"/>
-      <c r="M53" s="114"/>
-      <c r="N53" s="108">
+      <c r="L53" s="114"/>
+      <c r="M53" s="115"/>
+      <c r="N53" s="116">
         <v>200</v>
       </c>
-      <c r="O53" s="108"/>
-      <c r="P53" s="108"/>
-      <c r="Q53" s="108" t="s">
+      <c r="O53" s="116"/>
+      <c r="P53" s="116"/>
+      <c r="Q53" s="109" t="s">
         <v>176</v>
       </c>
-      <c r="R53" s="108"/>
-      <c r="S53" s="108"/>
-      <c r="T53" s="115" t="s">
+      <c r="R53" s="109"/>
+      <c r="S53" s="109"/>
+      <c r="T53" s="117" t="s">
         <v>181</v>
       </c>
-      <c r="U53" s="115"/>
-      <c r="V53" s="115"/>
-      <c r="W53" s="115"/>
+      <c r="U53" s="117"/>
+      <c r="V53" s="117"/>
+      <c r="W53" s="117"/>
     </row>
     <row r="54" ht="101" customHeight="1" spans="1:23">
       <c r="A54" s="107"/>
       <c r="B54" s="107"/>
       <c r="C54" s="108" t="s">
+        <v>178</v>
+      </c>
+      <c r="D54" s="109"/>
+      <c r="E54" s="109"/>
+      <c r="F54" s="109"/>
+      <c r="G54" s="109"/>
+      <c r="H54" s="110" t="s">
         <v>182</v>
       </c>
-      <c r="D54" s="108"/>
-      <c r="E54" s="108"/>
-      <c r="F54" s="108"/>
-      <c r="G54" s="108"/>
-      <c r="H54" s="109" t="s">
+      <c r="I54" s="111"/>
+      <c r="J54" s="112"/>
+      <c r="K54" s="113" t="s">
         <v>183</v>
       </c>
-      <c r="I54" s="110"/>
-      <c r="J54" s="111"/>
-      <c r="K54" s="112" t="s">
-        <v>180</v>
-      </c>
-      <c r="L54" s="113"/>
-      <c r="M54" s="114"/>
-      <c r="N54" s="108">
+      <c r="L54" s="114"/>
+      <c r="M54" s="115"/>
+      <c r="N54" s="116">
         <v>200</v>
       </c>
-      <c r="O54" s="108"/>
-      <c r="P54" s="108"/>
-      <c r="Q54" s="108" t="s">
-        <v>176</v>
-      </c>
-      <c r="R54" s="108"/>
-      <c r="S54" s="108"/>
-      <c r="T54" s="115" t="s">
+      <c r="O54" s="116"/>
+      <c r="P54" s="116"/>
+      <c r="Q54" s="109" t="s">
+        <v>184</v>
+      </c>
+      <c r="R54" s="109"/>
+      <c r="S54" s="109"/>
+      <c r="T54" s="117" t="s">
         <v>181</v>
       </c>
-      <c r="U54" s="115"/>
-      <c r="V54" s="115"/>
-      <c r="W54" s="115"/>
-    </row>
-    <row r="55" ht="65" customHeight="1" spans="1:23">
+      <c r="U54" s="117"/>
+      <c r="V54" s="117"/>
+      <c r="W54" s="117"/>
+    </row>
+    <row r="55" ht="101" customHeight="1" spans="1:23">
       <c r="A55" s="107"/>
       <c r="B55" s="107"/>
       <c r="C55" s="108" t="s">
-        <v>184</v>
-      </c>
-      <c r="D55" s="108"/>
-      <c r="E55" s="108"/>
-      <c r="F55" s="108"/>
-      <c r="G55" s="108"/>
-      <c r="H55" s="109" t="s">
-        <v>183</v>
-      </c>
-      <c r="I55" s="110"/>
-      <c r="J55" s="111"/>
-      <c r="K55" s="112" t="s">
         <v>185</v>
       </c>
-      <c r="L55" s="113"/>
-      <c r="M55" s="114"/>
-      <c r="N55" s="108">
+      <c r="D55" s="109"/>
+      <c r="E55" s="109"/>
+      <c r="F55" s="109"/>
+      <c r="G55" s="109"/>
+      <c r="H55" s="110" t="s">
+        <v>186</v>
+      </c>
+      <c r="I55" s="111"/>
+      <c r="J55" s="112"/>
+      <c r="K55" s="113" t="s">
+        <v>180</v>
+      </c>
+      <c r="L55" s="114"/>
+      <c r="M55" s="115"/>
+      <c r="N55" s="116">
         <v>200</v>
       </c>
-      <c r="O55" s="108"/>
-      <c r="P55" s="108"/>
-      <c r="Q55" s="108" t="s">
+      <c r="O55" s="116"/>
+      <c r="P55" s="116"/>
+      <c r="Q55" s="109" t="s">
         <v>176</v>
       </c>
-      <c r="R55" s="108"/>
-      <c r="S55" s="108"/>
-      <c r="T55" s="115" t="s">
+      <c r="R55" s="109"/>
+      <c r="S55" s="109"/>
+      <c r="T55" s="117" t="s">
         <v>181</v>
       </c>
-      <c r="U55" s="115"/>
-      <c r="V55" s="115"/>
-      <c r="W55" s="115"/>
-    </row>
-    <row r="56" ht="82" customHeight="1" spans="1:23">
+      <c r="U55" s="117"/>
+      <c r="V55" s="117"/>
+      <c r="W55" s="117"/>
+    </row>
+    <row r="56" ht="65" customHeight="1" spans="1:23">
       <c r="A56" s="107"/>
       <c r="B56" s="107"/>
       <c r="C56" s="108" t="s">
+        <v>187</v>
+      </c>
+      <c r="D56" s="109"/>
+      <c r="E56" s="109"/>
+      <c r="F56" s="109"/>
+      <c r="G56" s="109"/>
+      <c r="H56" s="110" t="s">
         <v>186</v>
       </c>
-      <c r="D56" s="108"/>
-      <c r="E56" s="108"/>
-      <c r="F56" s="108"/>
-      <c r="G56" s="108"/>
-      <c r="H56" s="109" t="s">
-        <v>187</v>
-      </c>
-      <c r="I56" s="110"/>
-      <c r="J56" s="111"/>
-      <c r="K56" s="112" t="s">
+      <c r="I56" s="111"/>
+      <c r="J56" s="112"/>
+      <c r="K56" s="113" t="s">
         <v>188</v>
       </c>
-      <c r="L56" s="113"/>
-      <c r="M56" s="114"/>
-      <c r="N56" s="108">
+      <c r="L56" s="114"/>
+      <c r="M56" s="115"/>
+      <c r="N56" s="116">
         <v>200</v>
       </c>
-      <c r="O56" s="108"/>
-      <c r="P56" s="108"/>
-      <c r="Q56" s="108" t="s">
+      <c r="O56" s="116"/>
+      <c r="P56" s="116"/>
+      <c r="Q56" s="109" t="s">
         <v>176</v>
       </c>
-      <c r="R56" s="108"/>
-      <c r="S56" s="108"/>
-      <c r="T56" s="115" t="s">
+      <c r="R56" s="109"/>
+      <c r="S56" s="109"/>
+      <c r="T56" s="117" t="s">
+        <v>181</v>
+      </c>
+      <c r="U56" s="117"/>
+      <c r="V56" s="117"/>
+      <c r="W56" s="117"/>
+    </row>
+    <row r="57" ht="82" customHeight="1" spans="1:23">
+      <c r="A57" s="107"/>
+      <c r="B57" s="107"/>
+      <c r="C57" s="108" t="s">
         <v>189</v>
       </c>
-      <c r="U56" s="115"/>
-      <c r="V56" s="115"/>
-      <c r="W56" s="115"/>
-    </row>
-    <row r="59" spans="1:23">
-      <c r="U59" s="15" t="s">
+      <c r="D57" s="109"/>
+      <c r="E57" s="109"/>
+      <c r="F57" s="109"/>
+      <c r="G57" s="109"/>
+      <c r="H57" s="110" t="s">
         <v>190</v>
       </c>
+      <c r="I57" s="111"/>
+      <c r="J57" s="112"/>
+      <c r="K57" s="113" t="s">
+        <v>191</v>
+      </c>
+      <c r="L57" s="114"/>
+      <c r="M57" s="115"/>
+      <c r="N57" s="116">
+        <v>200</v>
+      </c>
+      <c r="O57" s="116"/>
+      <c r="P57" s="116"/>
+      <c r="Q57" s="109" t="s">
+        <v>176</v>
+      </c>
+      <c r="R57" s="109"/>
+      <c r="S57" s="109"/>
+      <c r="T57" s="117" t="s">
+        <v>192</v>
+      </c>
+      <c r="U57" s="117"/>
+      <c r="V57" s="117"/>
+      <c r="W57" s="117"/>
+    </row>
+    <row r="58" ht="84" customHeight="1" spans="1:23">
+      <c r="A58" s="107"/>
+      <c r="B58" s="107"/>
+      <c r="C58" s="108" t="s">
+        <v>189</v>
+      </c>
+      <c r="D58" s="109"/>
+      <c r="E58" s="109"/>
+      <c r="F58" s="109"/>
+      <c r="G58" s="109"/>
+      <c r="H58" s="110" t="s">
+        <v>193</v>
+      </c>
+      <c r="I58" s="111"/>
+      <c r="J58" s="112"/>
+      <c r="K58" s="113" t="s">
+        <v>194</v>
+      </c>
+      <c r="L58" s="114"/>
+      <c r="M58" s="115"/>
+      <c r="N58" s="116">
+        <v>200</v>
+      </c>
+      <c r="O58" s="116"/>
+      <c r="P58" s="116"/>
+      <c r="Q58" s="109" t="s">
+        <v>184</v>
+      </c>
+      <c r="R58" s="109"/>
+      <c r="S58" s="109"/>
+      <c r="T58" s="117" t="s">
+        <v>195</v>
+      </c>
+      <c r="U58" s="117"/>
+      <c r="V58" s="117"/>
+      <c r="W58" s="117"/>
+    </row>
+    <row r="60" spans="1:23">
+      <c r="U60" s="15" t="s">
+        <v>196</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="292">
+  <mergeCells count="304">
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="A2:W2"/>
     <mergeCell ref="A3:B3"/>
@@ -4779,6 +4880,18 @@
     <mergeCell ref="N56:P56"/>
     <mergeCell ref="Q56:S56"/>
     <mergeCell ref="T56:W56"/>
+    <mergeCell ref="C57:G57"/>
+    <mergeCell ref="H57:J57"/>
+    <mergeCell ref="K57:M57"/>
+    <mergeCell ref="N57:P57"/>
+    <mergeCell ref="Q57:S57"/>
+    <mergeCell ref="T57:W57"/>
+    <mergeCell ref="C58:G58"/>
+    <mergeCell ref="H58:J58"/>
+    <mergeCell ref="K58:M58"/>
+    <mergeCell ref="N58:P58"/>
+    <mergeCell ref="Q58:S58"/>
+    <mergeCell ref="T58:W58"/>
     <mergeCell ref="A49:B50"/>
     <mergeCell ref="A45:B48"/>
     <mergeCell ref="A42:B43"/>
@@ -4797,7 +4910,7 @@
     <mergeCell ref="A10:B19"/>
     <mergeCell ref="T10:W16"/>
     <mergeCell ref="A21:B22"/>
-    <mergeCell ref="A52:B56"/>
+    <mergeCell ref="A52:B58"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C20" r:id="rId1" display="/api/v1/products/"/>
@@ -4821,7 +4934,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="B1" s="1" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -4836,45 +4949,45 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="2" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" s="6" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="B3" s="3">
         <v>1</v>
@@ -4912,7 +5025,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="6" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="B4" s="3">
         <v>1</v>
@@ -4950,7 +5063,7 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="6" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="B5" s="3">
         <v>1</v>
@@ -4988,7 +5101,7 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" s="6" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="B6" s="3">
         <v>1</v>
@@ -5026,7 +5139,7 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="6" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="B7" s="3">
         <v>1</v>
@@ -5064,7 +5177,7 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="10" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="11"/>
@@ -5080,7 +5193,7 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="6" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="B9" s="3">
         <v>1</v>
@@ -5088,23 +5201,23 @@
       <c r="C9" s="7">
         <v>1</v>
       </c>
-      <c r="D9" s="122" t="s">
-        <v>211</v>
-      </c>
-      <c r="E9" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="F9" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="G9" s="123" t="s">
-        <v>211</v>
+      <c r="D9" s="124" t="s">
+        <v>217</v>
+      </c>
+      <c r="E9" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="F9" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="G9" s="125" t="s">
+        <v>217</v>
       </c>
       <c r="H9" s="3">
         <v>1</v>
       </c>
-      <c r="I9" s="123" t="s">
-        <v>211</v>
+      <c r="I9" s="125" t="s">
+        <v>217</v>
       </c>
       <c r="J9" s="3">
         <v>1</v>
@@ -5112,31 +5225,31 @@
       <c r="K9" s="3">
         <v>1</v>
       </c>
-      <c r="L9" s="123" t="s">
-        <v>211</v>
+      <c r="L9" s="125" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="122" t="s">
-        <v>211</v>
+      <c r="C10" s="124" t="s">
+        <v>217</v>
       </c>
       <c r="D10" s="7">
         <v>1</v>
       </c>
-      <c r="E10" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="F10" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="G10" s="123" t="s">
-        <v>211</v>
+      <c r="E10" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="F10" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="G10" s="125" t="s">
+        <v>217</v>
       </c>
       <c r="H10" s="3">
         <v>1</v>
@@ -5144,125 +5257,125 @@
       <c r="I10" s="3">
         <v>1</v>
       </c>
-      <c r="J10" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="K10" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="L10" s="123" t="s">
-        <v>211</v>
+      <c r="J10" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="K10" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="L10" s="125" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="6" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B11" s="3">
         <v>1</v>
       </c>
-      <c r="C11" s="122" t="s">
-        <v>211</v>
-      </c>
-      <c r="D11" s="122" t="s">
-        <v>211</v>
+      <c r="C11" s="124" t="s">
+        <v>217</v>
+      </c>
+      <c r="D11" s="124" t="s">
+        <v>217</v>
       </c>
       <c r="E11" s="3">
         <v>1</v>
       </c>
-      <c r="F11" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="G11" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="H11" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="I11" s="123" t="s">
-        <v>211</v>
+      <c r="F11" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="G11" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="H11" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="I11" s="125" t="s">
+        <v>217</v>
       </c>
       <c r="J11" s="3">
         <v>1</v>
       </c>
-      <c r="K11" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="L11" s="123" t="s">
-        <v>211</v>
+      <c r="K11" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="L11" s="125" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="B12" s="3">
         <v>1</v>
       </c>
-      <c r="C12" s="122" t="s">
-        <v>211</v>
-      </c>
-      <c r="D12" s="122" t="s">
-        <v>211</v>
-      </c>
-      <c r="E12" s="123" t="s">
-        <v>211</v>
+      <c r="C12" s="124" t="s">
+        <v>217</v>
+      </c>
+      <c r="D12" s="124" t="s">
+        <v>217</v>
+      </c>
+      <c r="E12" s="125" t="s">
+        <v>217</v>
       </c>
       <c r="F12" s="3">
         <v>1</v>
       </c>
-      <c r="G12" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="H12" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="I12" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="J12" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="K12" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="L12" s="123" t="s">
-        <v>211</v>
+      <c r="G12" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="H12" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="I12" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="J12" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="K12" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="L12" s="125" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="6" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B13" s="3">
         <v>1</v>
       </c>
-      <c r="C13" s="122" t="s">
-        <v>211</v>
-      </c>
-      <c r="D13" s="122" t="s">
-        <v>211</v>
-      </c>
-      <c r="E13" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="F13" s="123" t="s">
-        <v>211</v>
+      <c r="C13" s="124" t="s">
+        <v>217</v>
+      </c>
+      <c r="D13" s="124" t="s">
+        <v>217</v>
+      </c>
+      <c r="E13" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="F13" s="125" t="s">
+        <v>217</v>
       </c>
       <c r="G13" s="3">
         <v>1</v>
       </c>
-      <c r="H13" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="I13" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="J13" s="123" t="s">
-        <v>211</v>
-      </c>
-      <c r="K13" s="123" t="s">
-        <v>211</v>
+      <c r="H13" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="I13" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="J13" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="K13" s="125" t="s">
+        <v>217</v>
       </c>
       <c r="L13" s="3">
         <v>1</v>
@@ -5278,14 +5391,14 @@
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
       <c r="I14" s="12" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="J14" s="13"/>
       <c r="K14" s="12" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="L14" s="12" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>